<commit_message>
Branch: NEXT-PRE-DEVELOPMENT - feat: add MadRock 27.5T product and update store inventory template
</commit_message>
<xml_diff>
--- a/store_inventory_template.xlsx
+++ b/store_inventory_template.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1001" uniqueCount="461">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1067" uniqueCount="460">
   <si>
     <t>category_id</t>
   </si>
@@ -29,115 +29,127 @@
     <t>description</t>
   </si>
   <si>
+    <t>brand</t>
+  </si>
+  <si>
     <t>seo_title</t>
   </si>
   <si>
-    <t>brand</t>
-  </si>
-  <si>
     <t>seo_description</t>
   </si>
   <si>
     <t>category_name</t>
   </si>
   <si>
+    <t>varient_label</t>
+  </si>
+  <si>
     <t>cat_001</t>
   </si>
   <si>
-    <t>varient_label</t>
+    <t>original_price</t>
   </si>
   <si>
     <t>Kids Cycle</t>
   </si>
   <si>
-    <t>original_price</t>
+    <t>discounted_price</t>
   </si>
   <si>
     <t>kids-cycle</t>
   </si>
   <si>
-    <t>discounted_price</t>
+    <t>discount_percent</t>
   </si>
   <si>
     <t>Kids Cycle available at KTR Cycle World, Tirunelveli.</t>
   </si>
   <si>
-    <t>discount_percent</t>
+    <t>stock</t>
   </si>
   <si>
     <t>Kids Cycle | KTR Cycle World</t>
   </si>
   <si>
-    <t>stock</t>
+    <t>featured</t>
+  </si>
+  <si>
+    <t>location</t>
   </si>
   <si>
     <t>cat_002</t>
   </si>
   <si>
-    <t>featured</t>
+    <t>color</t>
   </si>
   <si>
     <t>Adult Cycle</t>
   </si>
   <si>
-    <t>location</t>
+    <t>age_group</t>
   </si>
   <si>
     <t>adult-cycle</t>
   </si>
   <si>
-    <t>color</t>
+    <t>tags</t>
   </si>
   <si>
     <t>Adult Cycle available at KTR Cycle World, Tirunelveli.</t>
   </si>
   <si>
-    <t>age_group</t>
-  </si>
-  <si>
     <t>Adult Cycle | KTR Cycle World</t>
   </si>
   <si>
-    <t>tags</t>
+    <t>short_description</t>
+  </si>
+  <si>
+    <t>long_description</t>
   </si>
   <si>
     <t>cat_003</t>
   </si>
   <si>
-    <t>short_description</t>
-  </si>
-  <si>
     <t>Geared Cycle</t>
   </si>
   <si>
+    <t>specifications</t>
+  </si>
+  <si>
+    <t>features</t>
+  </si>
+  <si>
     <t>geared-cycle</t>
   </si>
   <si>
-    <t>long_description</t>
-  </si>
-  <si>
     <t>Geared Cycle available at KTR Cycle World, Tirunelveli.</t>
   </si>
   <si>
     <t>Geared Cycle | KTR Cycle World</t>
   </si>
   <si>
-    <t>specifications</t>
-  </si>
-  <si>
-    <t>features</t>
+    <t>images</t>
+  </si>
+  <si>
+    <t>prod_001</t>
   </si>
   <si>
     <t>cat_004</t>
   </si>
   <si>
+    <t>Alpha Bombay 26 VB</t>
+  </si>
+  <si>
     <t>Girls Cycle</t>
   </si>
   <si>
+    <t>alpha-bombay-26-vb</t>
+  </si>
+  <si>
     <t>girls-cycle</t>
   </si>
   <si>
-    <t>images</t>
+    <t>ALPHA</t>
   </si>
   <si>
     <t>Girls Cycle available at KTR Cycle World, Tirunelveli.</t>
@@ -146,69 +158,60 @@
     <t>Girls Cycle | KTR Cycle World</t>
   </si>
   <si>
-    <t>prod_001</t>
-  </si>
-  <si>
-    <t>Alpha Bombay 26 VB</t>
-  </si>
-  <si>
     <t>cat_005</t>
   </si>
   <si>
-    <t>alpha-bombay-26-vb</t>
-  </si>
-  <si>
     <t>Electric Cycle</t>
   </si>
   <si>
-    <t>ALPHA</t>
+    <t>FALSE</t>
   </si>
   <si>
     <t>electric-cycle</t>
   </si>
   <si>
+    <t>Tirunelveli</t>
+  </si>
+  <si>
     <t>Electric Cycle available at KTR Cycle World, Tirunelveli.</t>
   </si>
   <si>
+    <t>15+ Years</t>
+  </si>
+  <si>
     <t>Electric Cycle | KTR Cycle World</t>
   </si>
   <si>
+    <t>Alpha Bombay 26 VB - KTR Cycle World</t>
+  </si>
+  <si>
     <t>cat_006</t>
   </si>
   <si>
+    <t>/images/products/prod_001_1.jpg</t>
+  </si>
+  <si>
     <t>Offer cycle</t>
   </si>
   <si>
+    <t>prod_002</t>
+  </si>
+  <si>
     <t>offer-cycle</t>
   </si>
   <si>
+    <t>SKYWALK 20"</t>
+  </si>
+  <si>
     <t>Offer cycle available at KTR Cycle World, Tirunelveli.</t>
   </si>
   <si>
+    <t>skywalk-20</t>
+  </si>
+  <si>
     <t>Offer cycle | KTR Cycle World</t>
   </si>
   <si>
-    <t>FALSE</t>
-  </si>
-  <si>
-    <t>Tirunelveli</t>
-  </si>
-  <si>
-    <t>Alpha Bombay 26 VB - KTR Cycle World</t>
-  </si>
-  <si>
-    <t>/images/products/prod_001_1.jpg</t>
-  </si>
-  <si>
-    <t>prod_002</t>
-  </si>
-  <si>
-    <t>SKYWALK 20"</t>
-  </si>
-  <si>
-    <t>skywalk-20</t>
-  </si>
-  <si>
     <t>TORONTO</t>
   </si>
   <si>
@@ -218,6 +221,9 @@
     <t>TRUE</t>
   </si>
   <si>
+    <t>8-12 Years</t>
+  </si>
+  <si>
     <t>KIDS CYCLE</t>
   </si>
   <si>
@@ -275,7 +281,7 @@
     <t>Alpha cairo 24 FSDD</t>
   </si>
   <si>
-    <t xml:space="preserve">91 Alpha Cairo 24T D2TX 3.0 </t>
+    <t>12-15 Years</t>
   </si>
   <si>
     <t>91 Alpha Cairo 24T D2TX 3.0 - KTR Cycle World</t>
@@ -452,6 +458,9 @@
     <t>hercules</t>
   </si>
   <si>
+    <t>2-5 Years</t>
+  </si>
+  <si>
     <t>kids cycle for under 5 years</t>
   </si>
   <si>
@@ -488,6 +497,9 @@
     <t>bsa-champ-16t</t>
   </si>
   <si>
+    <t>5-8 Years</t>
+  </si>
+  <si>
     <t>kids cycle under 8 years</t>
   </si>
   <si>
@@ -944,9 +956,6 @@
     <t>hercules-rift-ic-fx-dd-24t</t>
   </si>
   <si>
-    <t xml:space="preserve">Hercules Rift IC FX DD 24T </t>
-  </si>
-  <si>
     <t>Hercules Rift IC FX DD 24T - KTR Cycle World</t>
   </si>
   <si>
@@ -962,9 +971,6 @@
     <t>hercules-rift-ic-fx-dd-26t</t>
   </si>
   <si>
-    <t xml:space="preserve">Hercules Rift IC FX DD 26T </t>
-  </si>
-  <si>
     <t>Hercules Rift IC FX DD 26T - KTR Cycle World</t>
   </si>
   <si>
@@ -980,9 +986,6 @@
     <t>hercules-rift-ic-rf-vb-24t</t>
   </si>
   <si>
-    <t xml:space="preserve">Hercules Rift IC RF VB 24T </t>
-  </si>
-  <si>
     <t>Hercules Rift IC RF VB 24T - KTR Cycle World</t>
   </si>
   <si>
@@ -1103,9 +1106,6 @@
     <t>SUNCROSS</t>
   </si>
   <si>
-    <t xml:space="preserve">HURRICANE 26T </t>
-  </si>
-  <si>
     <t>HURRICANE 26T - KTR Cycle World</t>
   </si>
   <si>
@@ -1244,9 +1244,6 @@
     <t>navarro-one</t>
   </si>
   <si>
-    <t xml:space="preserve">NAVARRO ONE </t>
-  </si>
-  <si>
     <t>NAVARRO ONE - KTR Cycle World</t>
   </si>
   <si>
@@ -1382,7 +1379,7 @@
     <t>MadRock 27.5T</t>
   </si>
   <si>
-    <t>madrock-27.5t</t>
+    <t>madrock-275t</t>
   </si>
   <si>
     <t>GEAR,ADULT</t>
@@ -1401,7 +1398,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <fonts count="4">
+  <fonts count="2">
     <font>
       <sz val="12.0"/>
       <color theme="1"/>
@@ -1412,17 +1409,6 @@
       <color theme="1"/>
       <name val="Calibri"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11.0"/>
-      <color rgb="FF9E9E9E"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="11.0"/>
-      <color rgb="FFE8E8E8"/>
-      <name val="Sans-serif"/>
     </font>
   </fonts>
   <fills count="2">
@@ -1439,18 +1425,11 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="2">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyFont="1"/>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle xfId="0" name="Normal" builtinId="0"/>
@@ -1687,8 +1666,7 @@
     <col customWidth="1" min="18" max="21" width="45.78"/>
     <col customWidth="1" min="22" max="22" width="35.78"/>
     <col customWidth="1" min="23" max="23" width="45.78"/>
-    <col customWidth="1" min="24" max="24" width="79.22"/>
-    <col customWidth="1" min="25" max="25" width="20.0"/>
+    <col customWidth="1" min="24" max="24" width="35.78"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1702,7 +1680,7 @@
         <v>3</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E1" s="1" t="s">
         <v>0</v>
@@ -1711,81 +1689,81 @@
         <v>8</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="L1" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="M1" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="N1" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="O1" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="P1" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="P1" s="1" t="s">
-        <v>28</v>
-      </c>
       <c r="Q1" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="R1" s="1" t="s">
         <v>30</v>
-      </c>
-      <c r="R1" s="1" t="s">
-        <v>33</v>
       </c>
       <c r="S1" s="1" t="s">
         <v>4</v>
       </c>
       <c r="T1" s="1" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="U1" s="1" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="V1" s="1" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="W1" s="1" t="s">
         <v>7</v>
       </c>
       <c r="X1" s="1" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="1" t="s">
-        <v>44</v>
+        <v>39</v>
       </c>
       <c r="B2" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="D2" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="C2" s="1" t="s">
-        <v>47</v>
-      </c>
-      <c r="D2" s="1" t="s">
-        <v>49</v>
-      </c>
       <c r="E2" s="1" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>45</v>
+        <v>41</v>
       </c>
       <c r="H2" s="1">
         <v>7200.0</v>
@@ -1800,45 +1778,48 @@
         <v>1.0</v>
       </c>
       <c r="L2" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="M2" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="O2" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="S2" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="V2" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="W2" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="X2" s="1" t="s">
         <v>58</v>
-      </c>
-      <c r="M2" s="1" t="s">
-        <v>59</v>
-      </c>
-      <c r="S2" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="V2" s="1" t="s">
-        <v>60</v>
-      </c>
-      <c r="W2" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="X2" s="1" t="s">
-        <v>61</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="B3" s="1" t="s">
         <v>62</v>
-      </c>
-      <c r="B3" s="1" t="s">
-        <v>63</v>
       </c>
       <c r="C3" s="1" t="s">
         <v>64</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="G3" s="1" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="H3" s="1">
         <v>11200.0</v>
@@ -1853,51 +1834,54 @@
         <v>3.0</v>
       </c>
       <c r="L3" s="1" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="M3" s="1" t="s">
-        <v>59</v>
+        <v>52</v>
+      </c>
+      <c r="O3" s="1" t="s">
+        <v>69</v>
       </c>
       <c r="P3" s="1" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="Q3" s="1" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="S3" s="1" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="V3" s="1" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="W3" s="1" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="X3" s="1" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="1" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F4" s="1" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="G4" s="1" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="H4" s="1">
         <v>11200.0</v>
@@ -1912,51 +1896,54 @@
         <v>3.0</v>
       </c>
       <c r="L4" s="1" t="s">
-        <v>58</v>
+        <v>50</v>
       </c>
       <c r="M4" s="1" t="s">
-        <v>59</v>
+        <v>52</v>
+      </c>
+      <c r="O4" s="1" t="s">
+        <v>69</v>
       </c>
       <c r="P4" s="1" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="Q4" s="1" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="S4" s="1" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="V4" s="1" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="W4" s="1" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="X4" s="1" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="1" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="D5" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="E5" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="F5" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="G5" s="1" t="s">
         <v>80</v>
-      </c>
-      <c r="E5" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="F5" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="G5" s="1" t="s">
-        <v>78</v>
       </c>
       <c r="H5" s="1">
         <v>6400.0</v>
@@ -1971,51 +1958,54 @@
         <v>3.0</v>
       </c>
       <c r="L5" s="1" t="s">
-        <v>58</v>
+        <v>50</v>
       </c>
       <c r="M5" s="1" t="s">
-        <v>59</v>
+        <v>52</v>
+      </c>
+      <c r="O5" s="1" t="s">
+        <v>69</v>
       </c>
       <c r="P5" s="1" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="Q5" s="1" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="S5" s="1" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="V5" s="1" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="W5" s="1" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="X5" s="1" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="1" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="F6" s="1" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="G6" s="1" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="H6" s="1">
         <v>10200.0</v>
@@ -2030,45 +2020,48 @@
         <v>1.0</v>
       </c>
       <c r="L6" s="1" t="s">
-        <v>58</v>
+        <v>50</v>
       </c>
       <c r="M6" s="1" t="s">
-        <v>59</v>
+        <v>52</v>
+      </c>
+      <c r="O6" s="1" t="s">
+        <v>89</v>
       </c>
       <c r="S6" s="1" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="V6" s="1" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="W6" s="1" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="X6" s="1" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="1" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="D7" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="E7" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="F7" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="G7" s="1" t="s">
         <v>93</v>
-      </c>
-      <c r="E7" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="F7" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="G7" s="1" t="s">
-        <v>91</v>
       </c>
       <c r="H7" s="1">
         <v>10400.0</v>
@@ -2083,51 +2076,54 @@
         <v>6.0</v>
       </c>
       <c r="L7" s="1" t="s">
-        <v>58</v>
+        <v>50</v>
       </c>
       <c r="M7" s="1" t="s">
-        <v>59</v>
+        <v>52</v>
+      </c>
+      <c r="O7" s="1" t="s">
+        <v>54</v>
       </c>
       <c r="P7" s="1" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="Q7" s="1" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="S7" s="1" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="V7" s="1" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="W7" s="1" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="X7" s="1" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="1" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="F8" s="1" t="s">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="G8" s="1" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="H8" s="1">
         <v>7800.0</v>
@@ -2142,48 +2138,51 @@
         <v>1.0</v>
       </c>
       <c r="L8" s="1" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="M8" s="1" t="s">
-        <v>59</v>
+        <v>52</v>
+      </c>
+      <c r="O8" s="1" t="s">
+        <v>54</v>
       </c>
       <c r="P8" s="1" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="S8" s="1" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="V8" s="1" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="W8" s="1" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="X8" s="1" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="1" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="E9" s="1" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="F9" s="1" t="s">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="G9" s="1" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="H9" s="1">
         <v>8500.0</v>
@@ -2198,48 +2197,51 @@
         <v>1.0</v>
       </c>
       <c r="L9" s="1" t="s">
-        <v>58</v>
+        <v>50</v>
       </c>
       <c r="M9" s="1" t="s">
-        <v>59</v>
+        <v>52</v>
+      </c>
+      <c r="O9" s="1" t="s">
+        <v>89</v>
       </c>
       <c r="P9" s="1" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="S9" s="1" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="V9" s="1" t="s">
+        <v>110</v>
+      </c>
+      <c r="W9" s="1" t="s">
         <v>108</v>
       </c>
-      <c r="W9" s="1" t="s">
-        <v>106</v>
-      </c>
       <c r="X9" s="1" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="1" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="D10" s="1" t="s">
+        <v>115</v>
+      </c>
+      <c r="E10" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="F10" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="G10" s="1" t="s">
         <v>113</v>
-      </c>
-      <c r="E10" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="F10" s="1" t="s">
-        <v>39</v>
-      </c>
-      <c r="G10" s="1" t="s">
-        <v>111</v>
       </c>
       <c r="H10" s="1">
         <v>7600.0</v>
@@ -2254,48 +2256,51 @@
         <v>3.0</v>
       </c>
       <c r="L10" s="1" t="s">
-        <v>58</v>
+        <v>50</v>
       </c>
       <c r="M10" s="1" t="s">
-        <v>59</v>
+        <v>52</v>
+      </c>
+      <c r="O10" s="1" t="s">
+        <v>54</v>
       </c>
       <c r="P10" s="1" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="S10" s="1" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="V10" s="1" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="W10" s="1" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="X10" s="1" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="1" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="E11" s="1" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="F11" s="1" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="G11" s="1" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="H11" s="1">
         <v>13500.0</v>
@@ -2310,51 +2315,54 @@
         <v>2.0</v>
       </c>
       <c r="L11" s="1" t="s">
-        <v>58</v>
+        <v>50</v>
       </c>
       <c r="M11" s="1" t="s">
-        <v>59</v>
+        <v>52</v>
+      </c>
+      <c r="O11" s="1" t="s">
+        <v>54</v>
       </c>
       <c r="P11" s="1" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="Q11" s="1" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="S11" s="1" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="V11" s="1" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="W11" s="1" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="X11" s="1" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="1" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="D12" s="1" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="E12" s="1" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F12" s="1" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="G12" s="1" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="H12" s="1">
         <v>7900.0</v>
@@ -2369,51 +2377,54 @@
         <v>2.0</v>
       </c>
       <c r="L12" s="1" t="s">
-        <v>58</v>
+        <v>50</v>
       </c>
       <c r="M12" s="1" t="s">
-        <v>59</v>
+        <v>52</v>
+      </c>
+      <c r="O12" s="1" t="s">
+        <v>69</v>
       </c>
       <c r="P12" s="1" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="Q12" s="1" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="S12" s="1" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="V12" s="1" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="W12" s="1" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="X12" s="1" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="1" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="D13" s="1" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="E13" s="1" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="F13" s="1" t="s">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="G13" s="1" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="H13" s="1">
         <v>7800.0</v>
@@ -2428,48 +2439,51 @@
         <v>4.0</v>
       </c>
       <c r="L13" s="1" t="s">
-        <v>58</v>
+        <v>50</v>
       </c>
       <c r="M13" s="1" t="s">
-        <v>59</v>
+        <v>52</v>
+      </c>
+      <c r="O13" s="1" t="s">
+        <v>89</v>
       </c>
       <c r="P13" s="1" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="S13" s="1" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="V13" s="1" t="s">
+        <v>134</v>
+      </c>
+      <c r="W13" s="1" t="s">
         <v>132</v>
       </c>
-      <c r="W13" s="1" t="s">
-        <v>130</v>
-      </c>
       <c r="X13" s="1" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="1" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="D14" s="1" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="E14" s="1" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="F14" s="1" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="G14" s="1" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="H14" s="1">
         <v>0.0</v>
@@ -2484,51 +2498,54 @@
         <v>0.0</v>
       </c>
       <c r="L14" s="1" t="s">
-        <v>58</v>
+        <v>50</v>
       </c>
       <c r="M14" s="1" t="s">
-        <v>59</v>
+        <v>52</v>
+      </c>
+      <c r="O14" s="1" t="s">
+        <v>54</v>
       </c>
       <c r="P14" s="1" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="Q14" s="1" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="S14" s="1" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="V14" s="1" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="W14" s="1" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="X14" s="1" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="1" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="D15" s="1" t="s">
+        <v>147</v>
+      </c>
+      <c r="E15" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="F15" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="G15" s="1" t="s">
         <v>145</v>
-      </c>
-      <c r="E15" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="F15" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="G15" s="1" t="s">
-        <v>143</v>
       </c>
       <c r="H15" s="1">
         <v>4400.0</v>
@@ -2543,51 +2560,54 @@
         <v>3.0</v>
       </c>
       <c r="L15" s="1" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="M15" s="1" t="s">
-        <v>59</v>
+        <v>52</v>
+      </c>
+      <c r="O15" s="1" t="s">
+        <v>148</v>
       </c>
       <c r="P15" s="1" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="Q15" s="1" t="s">
-        <v>146</v>
+        <v>149</v>
       </c>
       <c r="S15" s="1" t="s">
-        <v>146</v>
+        <v>149</v>
       </c>
       <c r="V15" s="1" t="s">
-        <v>147</v>
+        <v>150</v>
       </c>
       <c r="W15" s="1" t="s">
-        <v>146</v>
+        <v>149</v>
       </c>
       <c r="X15" s="1" t="s">
-        <v>148</v>
+        <v>151</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="1" t="s">
-        <v>149</v>
+        <v>152</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>150</v>
+        <v>153</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>151</v>
+        <v>154</v>
       </c>
       <c r="D16" s="1" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="E16" s="1" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F16" s="1" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="G16" s="1" t="s">
-        <v>150</v>
+        <v>153</v>
       </c>
       <c r="H16" s="1">
         <v>4500.0</v>
@@ -2602,51 +2622,54 @@
         <v>4.0</v>
       </c>
       <c r="L16" s="1" t="s">
-        <v>58</v>
+        <v>50</v>
       </c>
       <c r="M16" s="1" t="s">
-        <v>59</v>
+        <v>52</v>
+      </c>
+      <c r="O16" s="1" t="s">
+        <v>148</v>
       </c>
       <c r="P16" s="1" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="Q16" s="1" t="s">
-        <v>152</v>
+        <v>155</v>
       </c>
       <c r="S16" s="1" t="s">
-        <v>152</v>
+        <v>155</v>
       </c>
       <c r="V16" s="1" t="s">
-        <v>153</v>
+        <v>156</v>
       </c>
       <c r="W16" s="1" t="s">
-        <v>152</v>
+        <v>155</v>
       </c>
       <c r="X16" s="1" t="s">
-        <v>154</v>
+        <v>157</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="1" t="s">
-        <v>155</v>
+        <v>158</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>156</v>
+        <v>159</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="D17" s="1" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="E17" s="1" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F17" s="1" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="G17" s="1" t="s">
-        <v>156</v>
+        <v>159</v>
       </c>
       <c r="H17" s="1">
         <v>4900.0</v>
@@ -2661,51 +2684,54 @@
         <v>3.0</v>
       </c>
       <c r="L17" s="1" t="s">
-        <v>58</v>
+        <v>50</v>
       </c>
       <c r="M17" s="1" t="s">
-        <v>59</v>
+        <v>52</v>
+      </c>
+      <c r="O17" s="1" t="s">
+        <v>161</v>
       </c>
       <c r="P17" s="1" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="Q17" s="1" t="s">
-        <v>158</v>
+        <v>162</v>
       </c>
       <c r="S17" s="1" t="s">
-        <v>158</v>
+        <v>162</v>
       </c>
       <c r="V17" s="1" t="s">
-        <v>159</v>
+        <v>163</v>
       </c>
       <c r="W17" s="1" t="s">
-        <v>158</v>
+        <v>162</v>
       </c>
       <c r="X17" s="1" t="s">
-        <v>160</v>
+        <v>164</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="1" t="s">
-        <v>161</v>
+        <v>165</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>162</v>
+        <v>166</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>163</v>
+        <v>167</v>
       </c>
       <c r="D18" s="1" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="E18" s="1" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F18" s="1" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="G18" s="1" t="s">
-        <v>162</v>
+        <v>166</v>
       </c>
       <c r="H18" s="1">
         <v>5450.0</v>
@@ -2720,51 +2746,54 @@
         <v>5.0</v>
       </c>
       <c r="L18" s="1" t="s">
-        <v>58</v>
+        <v>50</v>
       </c>
       <c r="M18" s="1" t="s">
-        <v>59</v>
+        <v>52</v>
+      </c>
+      <c r="O18" s="1" t="s">
+        <v>69</v>
       </c>
       <c r="P18" s="1" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="Q18" s="1" t="s">
-        <v>164</v>
+        <v>168</v>
       </c>
       <c r="S18" s="1" t="s">
-        <v>164</v>
+        <v>168</v>
       </c>
       <c r="V18" s="1" t="s">
-        <v>165</v>
+        <v>169</v>
       </c>
       <c r="W18" s="1" t="s">
-        <v>164</v>
+        <v>168</v>
       </c>
       <c r="X18" s="1" t="s">
-        <v>166</v>
+        <v>170</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="1" t="s">
-        <v>167</v>
+        <v>171</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>168</v>
+        <v>172</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>169</v>
+        <v>173</v>
       </c>
       <c r="D19" s="1" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="E19" s="1" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F19" s="1" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="G19" s="1" t="s">
-        <v>168</v>
+        <v>172</v>
       </c>
       <c r="H19" s="1">
         <v>5300.0</v>
@@ -2779,48 +2808,51 @@
         <v>3.0</v>
       </c>
       <c r="L19" s="1" t="s">
-        <v>58</v>
+        <v>50</v>
       </c>
       <c r="M19" s="1" t="s">
-        <v>59</v>
+        <v>52</v>
+      </c>
+      <c r="O19" s="1" t="s">
+        <v>69</v>
       </c>
       <c r="P19" s="1" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="Q19" s="1" t="s">
-        <v>170</v>
+        <v>174</v>
       </c>
       <c r="S19" s="1" t="s">
-        <v>170</v>
+        <v>174</v>
       </c>
       <c r="V19" s="1" t="s">
-        <v>171</v>
+        <v>175</v>
       </c>
       <c r="W19" s="1" t="s">
-        <v>170</v>
+        <v>174</v>
       </c>
       <c r="X19" s="1" t="s">
-        <v>172</v>
+        <v>176</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="1" t="s">
-        <v>173</v>
+        <v>177</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>174</v>
+        <v>178</v>
       </c>
       <c r="C20" s="1" t="s">
-        <v>175</v>
+        <v>179</v>
       </c>
       <c r="E20" s="1" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="F20" s="1" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="G20" s="1" t="s">
-        <v>176</v>
+        <v>180</v>
       </c>
       <c r="H20" s="1">
         <v>8400.0</v>
@@ -2835,51 +2867,54 @@
         <v>2.0</v>
       </c>
       <c r="L20" s="1" t="s">
-        <v>58</v>
+        <v>50</v>
       </c>
       <c r="M20" s="1" t="s">
-        <v>59</v>
+        <v>52</v>
+      </c>
+      <c r="O20" s="1" t="s">
+        <v>54</v>
       </c>
       <c r="P20" s="1" t="s">
-        <v>177</v>
+        <v>181</v>
       </c>
       <c r="Q20" s="1" t="s">
-        <v>178</v>
+        <v>182</v>
       </c>
       <c r="S20" s="1" t="s">
-        <v>178</v>
+        <v>182</v>
       </c>
       <c r="V20" s="1" t="s">
-        <v>179</v>
+        <v>183</v>
       </c>
       <c r="W20" s="1" t="s">
-        <v>178</v>
+        <v>182</v>
       </c>
       <c r="X20" s="1" t="s">
-        <v>180</v>
+        <v>184</v>
       </c>
     </row>
     <row r="21" ht="15.75" customHeight="1">
       <c r="A21" s="1" t="s">
-        <v>181</v>
+        <v>185</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>182</v>
+        <v>186</v>
       </c>
       <c r="C21" s="1" t="s">
-        <v>183</v>
+        <v>187</v>
       </c>
       <c r="D21" s="1" t="s">
-        <v>184</v>
+        <v>188</v>
       </c>
       <c r="E21" s="1" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="F21" s="1" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="G21" s="1" t="s">
-        <v>182</v>
+        <v>186</v>
       </c>
       <c r="H21" s="1">
         <v>12500.0</v>
@@ -2894,48 +2929,51 @@
         <v>2.0</v>
       </c>
       <c r="L21" s="1" t="s">
-        <v>58</v>
+        <v>50</v>
       </c>
       <c r="M21" s="1" t="s">
-        <v>59</v>
+        <v>52</v>
+      </c>
+      <c r="O21" s="1" t="s">
+        <v>89</v>
       </c>
       <c r="P21" s="1" t="s">
-        <v>185</v>
+        <v>189</v>
       </c>
       <c r="S21" s="1" t="s">
-        <v>182</v>
+        <v>186</v>
       </c>
       <c r="V21" s="1" t="s">
+        <v>190</v>
+      </c>
+      <c r="W21" s="1" t="s">
         <v>186</v>
       </c>
-      <c r="W21" s="1" t="s">
-        <v>182</v>
-      </c>
       <c r="X21" s="1" t="s">
-        <v>187</v>
+        <v>191</v>
       </c>
     </row>
     <row r="22" ht="15.75" customHeight="1">
       <c r="A22" s="1" t="s">
-        <v>188</v>
+        <v>192</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>189</v>
+        <v>193</v>
       </c>
       <c r="C22" s="1" t="s">
-        <v>190</v>
+        <v>194</v>
       </c>
       <c r="D22" s="1" t="s">
-        <v>191</v>
+        <v>195</v>
       </c>
       <c r="E22" s="1" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="F22" s="1" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="G22" s="1" t="s">
-        <v>189</v>
+        <v>193</v>
       </c>
       <c r="H22" s="1">
         <v>38000.0</v>
@@ -2950,54 +2988,57 @@
         <v>3.0</v>
       </c>
       <c r="L22" s="1" t="s">
-        <v>58</v>
+        <v>50</v>
       </c>
       <c r="M22" s="1" t="s">
-        <v>59</v>
+        <v>52</v>
+      </c>
+      <c r="O22" s="1" t="s">
+        <v>54</v>
       </c>
       <c r="P22" s="1" t="s">
-        <v>192</v>
+        <v>196</v>
       </c>
       <c r="Q22" s="1" t="s">
-        <v>193</v>
+        <v>197</v>
       </c>
       <c r="R22" s="1" t="s">
-        <v>194</v>
+        <v>198</v>
       </c>
       <c r="S22" s="1" t="s">
-        <v>194</v>
+        <v>198</v>
       </c>
       <c r="V22" s="1" t="s">
-        <v>195</v>
+        <v>199</v>
       </c>
       <c r="W22" s="1" t="s">
-        <v>193</v>
+        <v>197</v>
       </c>
       <c r="X22" s="1" t="s">
-        <v>196</v>
+        <v>200</v>
       </c>
     </row>
     <row r="23" ht="15.75" customHeight="1">
       <c r="A23" s="1" t="s">
-        <v>197</v>
+        <v>201</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>198</v>
+        <v>202</v>
       </c>
       <c r="C23" s="1" t="s">
-        <v>199</v>
+        <v>203</v>
       </c>
       <c r="D23" s="1" t="s">
-        <v>200</v>
+        <v>204</v>
       </c>
       <c r="E23" s="1" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="F23" s="1" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="G23" s="1" t="s">
-        <v>200</v>
+        <v>204</v>
       </c>
       <c r="H23" s="1">
         <v>24000.0</v>
@@ -3012,51 +3053,54 @@
         <v>3.0</v>
       </c>
       <c r="L23" s="1" t="s">
-        <v>58</v>
+        <v>50</v>
       </c>
       <c r="M23" s="1" t="s">
-        <v>59</v>
+        <v>52</v>
+      </c>
+      <c r="O23" s="1" t="s">
+        <v>54</v>
       </c>
       <c r="P23" s="1" t="s">
-        <v>192</v>
+        <v>196</v>
       </c>
       <c r="Q23" s="1" t="s">
-        <v>201</v>
+        <v>205</v>
       </c>
       <c r="R23" s="1" t="s">
-        <v>202</v>
+        <v>206</v>
       </c>
       <c r="S23" s="1" t="s">
-        <v>202</v>
+        <v>206</v>
       </c>
       <c r="V23" s="1" t="s">
-        <v>203</v>
+        <v>207</v>
       </c>
       <c r="W23" s="1" t="s">
-        <v>201</v>
+        <v>205</v>
       </c>
       <c r="X23" s="1" t="s">
-        <v>204</v>
+        <v>208</v>
       </c>
     </row>
     <row r="24" ht="15.75" customHeight="1">
       <c r="A24" s="1" t="s">
-        <v>205</v>
+        <v>209</v>
       </c>
       <c r="B24" s="1" t="s">
-        <v>206</v>
+        <v>210</v>
       </c>
       <c r="C24" s="1" t="s">
-        <v>207</v>
+        <v>211</v>
       </c>
       <c r="E24" s="1" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="F24" s="1" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="G24" s="1" t="s">
-        <v>208</v>
+        <v>212</v>
       </c>
       <c r="H24" s="1">
         <v>12500.0</v>
@@ -3071,42 +3115,45 @@
         <v>1.0</v>
       </c>
       <c r="L24" s="1" t="s">
-        <v>58</v>
+        <v>50</v>
       </c>
       <c r="M24" s="1" t="s">
-        <v>59</v>
+        <v>52</v>
+      </c>
+      <c r="O24" s="1" t="s">
+        <v>54</v>
       </c>
       <c r="S24" s="1" t="s">
-        <v>206</v>
+        <v>210</v>
       </c>
       <c r="V24" s="1" t="s">
-        <v>209</v>
+        <v>213</v>
       </c>
       <c r="W24" s="1" t="s">
-        <v>206</v>
+        <v>210</v>
       </c>
       <c r="X24" s="1" t="s">
-        <v>210</v>
+        <v>214</v>
       </c>
     </row>
     <row r="25" ht="15.75" customHeight="1">
       <c r="A25" s="1" t="s">
-        <v>211</v>
+        <v>215</v>
       </c>
       <c r="B25" s="1" t="s">
-        <v>212</v>
+        <v>216</v>
       </c>
       <c r="C25" s="1" t="s">
-        <v>213</v>
+        <v>217</v>
       </c>
       <c r="E25" s="1" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="F25" s="1" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="G25" s="1" t="s">
-        <v>214</v>
+        <v>218</v>
       </c>
       <c r="H25" s="1">
         <v>14175.0</v>
@@ -3121,51 +3168,54 @@
         <v>1.0</v>
       </c>
       <c r="L25" s="1" t="s">
-        <v>58</v>
+        <v>50</v>
       </c>
       <c r="M25" s="1" t="s">
-        <v>59</v>
+        <v>52</v>
+      </c>
+      <c r="O25" s="1" t="s">
+        <v>54</v>
       </c>
       <c r="P25" s="1" t="s">
-        <v>215</v>
+        <v>219</v>
       </c>
       <c r="Q25" s="1" t="s">
-        <v>216</v>
+        <v>220</v>
       </c>
       <c r="S25" s="1" t="s">
-        <v>216</v>
+        <v>220</v>
       </c>
       <c r="V25" s="1" t="s">
-        <v>217</v>
+        <v>221</v>
       </c>
       <c r="W25" s="1" t="s">
-        <v>216</v>
+        <v>220</v>
       </c>
       <c r="X25" s="1" t="s">
-        <v>218</v>
+        <v>222</v>
       </c>
     </row>
     <row r="26" ht="15.75" customHeight="1">
       <c r="A26" s="1" t="s">
-        <v>219</v>
+        <v>223</v>
       </c>
       <c r="B26" s="1" t="s">
-        <v>220</v>
+        <v>224</v>
       </c>
       <c r="C26" s="1" t="s">
-        <v>221</v>
+        <v>225</v>
       </c>
       <c r="D26" s="1" t="s">
-        <v>200</v>
+        <v>204</v>
       </c>
       <c r="E26" s="1" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="F26" s="1" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="G26" s="1" t="s">
-        <v>200</v>
+        <v>204</v>
       </c>
       <c r="H26" s="1">
         <v>31000.0</v>
@@ -3180,51 +3230,54 @@
         <v>3.0</v>
       </c>
       <c r="L26" s="1" t="s">
-        <v>58</v>
+        <v>50</v>
       </c>
       <c r="M26" s="1" t="s">
-        <v>59</v>
+        <v>52</v>
+      </c>
+      <c r="O26" s="1" t="s">
+        <v>54</v>
       </c>
       <c r="P26" s="1" t="s">
-        <v>192</v>
+        <v>196</v>
       </c>
       <c r="Q26" s="1" t="s">
-        <v>222</v>
+        <v>226</v>
       </c>
       <c r="R26" s="1" t="s">
-        <v>223</v>
+        <v>227</v>
       </c>
       <c r="S26" s="1" t="s">
-        <v>223</v>
+        <v>227</v>
       </c>
       <c r="V26" s="1" t="s">
-        <v>224</v>
+        <v>228</v>
       </c>
       <c r="W26" s="1" t="s">
-        <v>222</v>
+        <v>226</v>
       </c>
       <c r="X26" s="1" t="s">
-        <v>225</v>
+        <v>229</v>
       </c>
     </row>
     <row r="27" ht="15.75" customHeight="1">
       <c r="A27" s="1" t="s">
-        <v>226</v>
+        <v>230</v>
       </c>
       <c r="B27" s="1" t="s">
-        <v>227</v>
+        <v>231</v>
       </c>
       <c r="C27" s="1" t="s">
-        <v>228</v>
+        <v>232</v>
       </c>
       <c r="E27" s="1" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="F27" s="1" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="G27" s="1" t="s">
-        <v>229</v>
+        <v>233</v>
       </c>
       <c r="H27" s="1">
         <v>9999.0</v>
@@ -3239,48 +3292,51 @@
         <v>1.0</v>
       </c>
       <c r="L27" s="1" t="s">
-        <v>58</v>
+        <v>50</v>
       </c>
       <c r="M27" s="1" t="s">
-        <v>59</v>
+        <v>52</v>
       </c>
       <c r="N27" s="1" t="s">
-        <v>230</v>
+        <v>234</v>
+      </c>
+      <c r="O27" s="1" t="s">
+        <v>54</v>
       </c>
       <c r="Q27" s="1" t="s">
-        <v>231</v>
+        <v>235</v>
       </c>
       <c r="S27" s="1" t="s">
-        <v>231</v>
+        <v>235</v>
       </c>
       <c r="V27" s="1" t="s">
-        <v>232</v>
+        <v>236</v>
       </c>
       <c r="W27" s="1" t="s">
-        <v>231</v>
+        <v>235</v>
       </c>
       <c r="X27" s="1" t="s">
-        <v>233</v>
+        <v>237</v>
       </c>
     </row>
     <row r="28" ht="15.75" customHeight="1">
       <c r="A28" s="1" t="s">
-        <v>234</v>
+        <v>238</v>
       </c>
       <c r="B28" s="1" t="s">
-        <v>235</v>
+        <v>239</v>
       </c>
       <c r="C28" s="1" t="s">
-        <v>236</v>
+        <v>240</v>
       </c>
       <c r="E28" s="1" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="F28" s="1" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="G28" s="1" t="s">
-        <v>235</v>
+        <v>239</v>
       </c>
       <c r="H28" s="1">
         <v>20400.0</v>
@@ -3295,48 +3351,51 @@
         <v>2.0</v>
       </c>
       <c r="L28" s="1" t="s">
-        <v>58</v>
+        <v>50</v>
       </c>
       <c r="M28" s="1" t="s">
-        <v>59</v>
+        <v>52</v>
+      </c>
+      <c r="O28" s="1" t="s">
+        <v>54</v>
       </c>
       <c r="P28" s="1" t="s">
-        <v>237</v>
+        <v>241</v>
       </c>
       <c r="S28" s="1" t="s">
-        <v>235</v>
+        <v>239</v>
       </c>
       <c r="V28" s="1" t="s">
-        <v>238</v>
+        <v>242</v>
       </c>
       <c r="W28" s="1" t="s">
-        <v>235</v>
+        <v>239</v>
       </c>
       <c r="X28" s="1" t="s">
-        <v>239</v>
+        <v>243</v>
       </c>
     </row>
     <row r="29" ht="15.75" customHeight="1">
       <c r="A29" s="1" t="s">
-        <v>240</v>
+        <v>244</v>
       </c>
       <c r="B29" s="1" t="s">
-        <v>241</v>
+        <v>245</v>
       </c>
       <c r="C29" s="1" t="s">
-        <v>242</v>
+        <v>246</v>
       </c>
       <c r="D29" s="1" t="s">
-        <v>243</v>
+        <v>247</v>
       </c>
       <c r="E29" s="1" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="F29" s="1" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="G29" s="1" t="s">
-        <v>241</v>
+        <v>245</v>
       </c>
       <c r="H29" s="1">
         <v>19000.0</v>
@@ -3351,51 +3410,54 @@
         <v>3.0</v>
       </c>
       <c r="L29" s="1" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="M29" s="1" t="s">
-        <v>59</v>
+        <v>52</v>
+      </c>
+      <c r="O29" s="1" t="s">
+        <v>54</v>
       </c>
       <c r="P29" s="1" t="s">
-        <v>244</v>
+        <v>248</v>
       </c>
       <c r="Q29" s="1" t="s">
-        <v>245</v>
+        <v>249</v>
       </c>
       <c r="S29" s="1" t="s">
-        <v>245</v>
+        <v>249</v>
       </c>
       <c r="V29" s="1" t="s">
-        <v>246</v>
+        <v>250</v>
       </c>
       <c r="W29" s="1" t="s">
-        <v>245</v>
+        <v>249</v>
       </c>
       <c r="X29" s="1" t="s">
-        <v>247</v>
+        <v>251</v>
       </c>
     </row>
     <row r="30" ht="15.75" customHeight="1">
       <c r="A30" s="1" t="s">
-        <v>248</v>
+        <v>252</v>
       </c>
       <c r="B30" s="1" t="s">
-        <v>249</v>
+        <v>253</v>
       </c>
       <c r="C30" s="1" t="s">
-        <v>250</v>
+        <v>254</v>
       </c>
       <c r="D30" s="1" t="s">
-        <v>251</v>
+        <v>255</v>
       </c>
       <c r="E30" s="1" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="F30" s="1" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="G30" s="1" t="s">
-        <v>251</v>
+        <v>255</v>
       </c>
       <c r="H30" s="1">
         <v>29900.0</v>
@@ -3410,54 +3472,57 @@
         <v>3.0</v>
       </c>
       <c r="L30" s="1" t="s">
-        <v>58</v>
+        <v>50</v>
       </c>
       <c r="M30" s="1" t="s">
-        <v>59</v>
+        <v>52</v>
+      </c>
+      <c r="O30" s="1" t="s">
+        <v>54</v>
       </c>
       <c r="P30" s="1" t="s">
-        <v>192</v>
+        <v>196</v>
       </c>
       <c r="Q30" s="1" t="s">
-        <v>252</v>
+        <v>256</v>
       </c>
       <c r="R30" s="1" t="s">
-        <v>253</v>
+        <v>257</v>
       </c>
       <c r="S30" s="1" t="s">
-        <v>253</v>
+        <v>257</v>
       </c>
       <c r="V30" s="1" t="s">
-        <v>254</v>
+        <v>258</v>
       </c>
       <c r="W30" s="1" t="s">
-        <v>252</v>
+        <v>256</v>
       </c>
       <c r="X30" s="1" t="s">
-        <v>255</v>
+        <v>259</v>
       </c>
     </row>
     <row r="31" ht="15.75" customHeight="1">
       <c r="A31" s="1" t="s">
-        <v>256</v>
+        <v>260</v>
       </c>
       <c r="B31" s="1" t="s">
-        <v>257</v>
+        <v>261</v>
       </c>
       <c r="C31" s="1" t="s">
-        <v>258</v>
+        <v>262</v>
       </c>
       <c r="D31" s="1" t="s">
-        <v>259</v>
+        <v>263</v>
       </c>
       <c r="E31" s="1" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F31" s="1" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="G31" s="1" t="s">
-        <v>259</v>
+        <v>263</v>
       </c>
       <c r="H31" s="1">
         <v>5200.0</v>
@@ -3472,48 +3537,51 @@
         <v>5.0</v>
       </c>
       <c r="L31" s="1" t="s">
-        <v>58</v>
+        <v>50</v>
       </c>
       <c r="M31" s="1" t="s">
-        <v>59</v>
+        <v>52</v>
+      </c>
+      <c r="O31" s="1" t="s">
+        <v>69</v>
       </c>
       <c r="P31" s="1" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="S31" s="1" t="s">
-        <v>257</v>
+        <v>261</v>
       </c>
       <c r="V31" s="1" t="s">
-        <v>260</v>
+        <v>264</v>
       </c>
       <c r="W31" s="1" t="s">
-        <v>257</v>
+        <v>261</v>
       </c>
       <c r="X31" s="1" t="s">
-        <v>261</v>
+        <v>265</v>
       </c>
     </row>
     <row r="32" ht="15.75" customHeight="1">
       <c r="A32" s="1" t="s">
-        <v>262</v>
+        <v>266</v>
       </c>
       <c r="B32" s="1" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
       <c r="C32" s="1" t="s">
-        <v>264</v>
+        <v>268</v>
       </c>
       <c r="D32" s="1" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="E32" s="1" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F32" s="1" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="G32" s="1" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="H32" s="1">
         <v>7200.0</v>
@@ -3528,48 +3596,51 @@
         <v>3.0</v>
       </c>
       <c r="L32" s="1" t="s">
-        <v>58</v>
+        <v>50</v>
       </c>
       <c r="M32" s="1" t="s">
-        <v>59</v>
+        <v>52</v>
+      </c>
+      <c r="O32" s="1" t="s">
+        <v>69</v>
       </c>
       <c r="P32" s="1" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="S32" s="1" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
       <c r="V32" s="1" t="s">
-        <v>265</v>
+        <v>269</v>
       </c>
       <c r="W32" s="1" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
       <c r="X32" s="1" t="s">
-        <v>266</v>
+        <v>270</v>
       </c>
     </row>
     <row r="33" ht="15.75" customHeight="1">
       <c r="A33" s="1" t="s">
-        <v>267</v>
+        <v>271</v>
       </c>
       <c r="B33" s="1" t="s">
-        <v>268</v>
+        <v>272</v>
       </c>
       <c r="C33" s="1" t="s">
-        <v>269</v>
+        <v>273</v>
       </c>
       <c r="D33" s="1" t="s">
-        <v>251</v>
+        <v>255</v>
       </c>
       <c r="E33" s="1" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="F33" s="1" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="G33" s="1" t="s">
-        <v>251</v>
+        <v>255</v>
       </c>
       <c r="H33" s="1">
         <v>27500.0</v>
@@ -3584,54 +3655,57 @@
         <v>3.0</v>
       </c>
       <c r="L33" s="1" t="s">
-        <v>58</v>
+        <v>50</v>
       </c>
       <c r="M33" s="1" t="s">
-        <v>59</v>
+        <v>52</v>
+      </c>
+      <c r="O33" s="1" t="s">
+        <v>54</v>
       </c>
       <c r="P33" s="1" t="s">
-        <v>192</v>
+        <v>196</v>
       </c>
       <c r="Q33" s="1" t="s">
-        <v>270</v>
+        <v>274</v>
       </c>
       <c r="R33" s="1" t="s">
-        <v>271</v>
+        <v>275</v>
       </c>
       <c r="S33" s="1" t="s">
-        <v>271</v>
+        <v>275</v>
       </c>
       <c r="V33" s="1" t="s">
-        <v>272</v>
+        <v>276</v>
       </c>
       <c r="W33" s="1" t="s">
-        <v>270</v>
+        <v>274</v>
       </c>
       <c r="X33" s="1" t="s">
-        <v>273</v>
+        <v>277</v>
       </c>
     </row>
     <row r="34" ht="15.75" customHeight="1">
       <c r="A34" s="1" t="s">
-        <v>274</v>
+        <v>278</v>
       </c>
       <c r="B34" s="1" t="s">
-        <v>275</v>
+        <v>279</v>
       </c>
       <c r="C34" s="1" t="s">
-        <v>276</v>
+        <v>280</v>
       </c>
       <c r="D34" s="1" t="s">
-        <v>251</v>
+        <v>255</v>
       </c>
       <c r="E34" s="1" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="F34" s="1" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="G34" s="1" t="s">
-        <v>251</v>
+        <v>255</v>
       </c>
       <c r="H34" s="1">
         <v>13500.0</v>
@@ -3646,48 +3720,51 @@
         <v>2.0</v>
       </c>
       <c r="L34" s="1" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="M34" s="1" t="s">
-        <v>59</v>
+        <v>52</v>
+      </c>
+      <c r="O34" s="1" t="s">
+        <v>54</v>
       </c>
       <c r="P34" s="1" t="s">
-        <v>277</v>
+        <v>281</v>
       </c>
       <c r="S34" s="1" t="s">
-        <v>275</v>
+        <v>279</v>
       </c>
       <c r="V34" s="1" t="s">
-        <v>278</v>
+        <v>282</v>
       </c>
       <c r="W34" s="1" t="s">
-        <v>275</v>
+        <v>279</v>
       </c>
       <c r="X34" s="1" t="s">
-        <v>279</v>
+        <v>283</v>
       </c>
     </row>
     <row r="35" ht="15.75" customHeight="1">
       <c r="A35" s="1" t="s">
-        <v>280</v>
+        <v>284</v>
       </c>
       <c r="B35" s="1" t="s">
-        <v>281</v>
+        <v>285</v>
       </c>
       <c r="C35" s="1" t="s">
-        <v>282</v>
+        <v>286</v>
       </c>
       <c r="D35" s="1" t="s">
-        <v>251</v>
+        <v>255</v>
       </c>
       <c r="E35" s="1" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="F35" s="1" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="G35" s="1" t="s">
-        <v>251</v>
+        <v>255</v>
       </c>
       <c r="H35" s="1">
         <v>6800.0</v>
@@ -3702,48 +3779,51 @@
         <v>3.0</v>
       </c>
       <c r="L35" s="1" t="s">
-        <v>58</v>
+        <v>50</v>
       </c>
       <c r="M35" s="1" t="s">
-        <v>59</v>
+        <v>52</v>
+      </c>
+      <c r="O35" s="1" t="s">
+        <v>54</v>
       </c>
       <c r="P35" s="1" t="s">
-        <v>283</v>
+        <v>287</v>
       </c>
       <c r="S35" s="1" t="s">
-        <v>281</v>
+        <v>285</v>
       </c>
       <c r="V35" s="1" t="s">
-        <v>284</v>
+        <v>288</v>
       </c>
       <c r="W35" s="1" t="s">
-        <v>281</v>
+        <v>285</v>
       </c>
       <c r="X35" s="1" t="s">
-        <v>285</v>
+        <v>289</v>
       </c>
     </row>
     <row r="36" ht="15.75" customHeight="1">
       <c r="A36" s="1" t="s">
-        <v>286</v>
+        <v>290</v>
       </c>
       <c r="B36" s="1" t="s">
-        <v>287</v>
+        <v>291</v>
       </c>
       <c r="C36" s="1" t="s">
-        <v>288</v>
+        <v>292</v>
       </c>
       <c r="D36" s="1" t="s">
-        <v>289</v>
+        <v>293</v>
       </c>
       <c r="E36" s="1" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F36" s="1" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="G36" s="1" t="s">
-        <v>289</v>
+        <v>293</v>
       </c>
       <c r="H36" s="1">
         <v>3500.0</v>
@@ -3758,48 +3838,51 @@
         <v>3.0</v>
       </c>
       <c r="L36" s="1" t="s">
-        <v>58</v>
+        <v>50</v>
       </c>
       <c r="M36" s="1" t="s">
-        <v>59</v>
+        <v>52</v>
+      </c>
+      <c r="O36" s="1" t="s">
+        <v>148</v>
       </c>
       <c r="P36" s="1" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="S36" s="1" t="s">
-        <v>287</v>
+        <v>291</v>
       </c>
       <c r="V36" s="1" t="s">
-        <v>290</v>
+        <v>294</v>
       </c>
       <c r="W36" s="1" t="s">
-        <v>287</v>
+        <v>291</v>
       </c>
       <c r="X36" s="1" t="s">
-        <v>291</v>
+        <v>295</v>
       </c>
     </row>
     <row r="37" ht="15.75" customHeight="1">
       <c r="A37" s="1" t="s">
-        <v>292</v>
+        <v>296</v>
       </c>
       <c r="B37" s="1" t="s">
+        <v>297</v>
+      </c>
+      <c r="C37" s="1" t="s">
+        <v>298</v>
+      </c>
+      <c r="D37" s="1" t="s">
         <v>293</v>
       </c>
-      <c r="C37" s="1" t="s">
-        <v>294</v>
-      </c>
-      <c r="D37" s="1" t="s">
-        <v>289</v>
-      </c>
       <c r="E37" s="1" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F37" s="1" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="G37" s="1" t="s">
-        <v>289</v>
+        <v>293</v>
       </c>
       <c r="H37" s="1">
         <v>4200.0</v>
@@ -3814,48 +3897,51 @@
         <v>3.0</v>
       </c>
       <c r="L37" s="1" t="s">
-        <v>58</v>
+        <v>50</v>
       </c>
       <c r="M37" s="1" t="s">
-        <v>59</v>
+        <v>52</v>
+      </c>
+      <c r="O37" s="1" t="s">
+        <v>69</v>
       </c>
       <c r="P37" s="1" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="S37" s="1" t="s">
-        <v>293</v>
+        <v>297</v>
       </c>
       <c r="V37" s="1" t="s">
-        <v>295</v>
+        <v>299</v>
       </c>
       <c r="W37" s="1" t="s">
-        <v>293</v>
+        <v>297</v>
       </c>
       <c r="X37" s="1" t="s">
-        <v>296</v>
+        <v>300</v>
       </c>
     </row>
     <row r="38" ht="15.75" customHeight="1">
       <c r="A38" s="1" t="s">
-        <v>297</v>
+        <v>301</v>
       </c>
       <c r="B38" s="1" t="s">
-        <v>298</v>
+        <v>302</v>
       </c>
       <c r="C38" s="1" t="s">
-        <v>299</v>
+        <v>303</v>
       </c>
       <c r="D38" s="1" t="s">
-        <v>289</v>
+        <v>293</v>
       </c>
       <c r="E38" s="1" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F38" s="1" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="G38" s="1" t="s">
-        <v>289</v>
+        <v>293</v>
       </c>
       <c r="H38" s="1">
         <v>3600.0</v>
@@ -3870,48 +3956,51 @@
         <v>3.0</v>
       </c>
       <c r="L38" s="1" t="s">
-        <v>58</v>
+        <v>50</v>
       </c>
       <c r="M38" s="1" t="s">
-        <v>59</v>
+        <v>52</v>
+      </c>
+      <c r="O38" s="1" t="s">
+        <v>161</v>
       </c>
       <c r="P38" s="1" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="S38" s="1" t="s">
-        <v>298</v>
+        <v>302</v>
       </c>
       <c r="V38" s="1" t="s">
-        <v>300</v>
+        <v>304</v>
       </c>
       <c r="W38" s="1" t="s">
-        <v>298</v>
+        <v>302</v>
       </c>
       <c r="X38" s="1" t="s">
-        <v>301</v>
+        <v>305</v>
       </c>
     </row>
     <row r="39" ht="15.75" customHeight="1">
       <c r="A39" s="1" t="s">
-        <v>302</v>
+        <v>306</v>
       </c>
       <c r="B39" s="1" t="s">
-        <v>303</v>
+        <v>307</v>
       </c>
       <c r="C39" s="1" t="s">
-        <v>304</v>
+        <v>308</v>
       </c>
       <c r="D39" s="1" t="s">
-        <v>251</v>
+        <v>255</v>
       </c>
       <c r="E39" s="1" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="F39" s="1" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="G39" s="1" t="s">
-        <v>251</v>
+        <v>255</v>
       </c>
       <c r="H39" s="1">
         <v>8200.0</v>
@@ -3926,48 +4015,51 @@
         <v>3.0</v>
       </c>
       <c r="L39" s="1" t="s">
-        <v>58</v>
+        <v>50</v>
       </c>
       <c r="M39" s="1" t="s">
-        <v>59</v>
+        <v>52</v>
+      </c>
+      <c r="O39" s="1" t="s">
+        <v>54</v>
       </c>
       <c r="P39" s="1" t="s">
-        <v>283</v>
+        <v>287</v>
       </c>
       <c r="S39" s="1" t="s">
-        <v>303</v>
+        <v>307</v>
       </c>
       <c r="V39" s="1" t="s">
-        <v>305</v>
+        <v>309</v>
       </c>
       <c r="W39" s="1" t="s">
-        <v>303</v>
+        <v>307</v>
       </c>
       <c r="X39" s="1" t="s">
-        <v>306</v>
+        <v>310</v>
       </c>
     </row>
     <row r="40" ht="15.75" customHeight="1">
       <c r="A40" s="1" t="s">
-        <v>307</v>
+        <v>311</v>
       </c>
       <c r="B40" s="1" t="s">
-        <v>308</v>
+        <v>312</v>
       </c>
       <c r="C40" s="1" t="s">
-        <v>309</v>
+        <v>313</v>
       </c>
       <c r="D40" s="1" t="s">
-        <v>251</v>
+        <v>255</v>
       </c>
       <c r="E40" s="1" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="F40" s="1" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="G40" s="1" t="s">
-        <v>251</v>
+        <v>255</v>
       </c>
       <c r="H40" s="1">
         <v>8100.0</v>
@@ -3982,48 +4074,51 @@
         <v>3.0</v>
       </c>
       <c r="L40" s="1" t="s">
-        <v>58</v>
+        <v>50</v>
       </c>
       <c r="M40" s="1" t="s">
-        <v>59</v>
+        <v>52</v>
+      </c>
+      <c r="O40" s="1" t="s">
+        <v>89</v>
       </c>
       <c r="P40" s="1" t="s">
-        <v>283</v>
+        <v>287</v>
       </c>
       <c r="S40" s="1" t="s">
-        <v>310</v>
+        <v>312</v>
       </c>
       <c r="V40" s="1" t="s">
-        <v>311</v>
+        <v>314</v>
       </c>
       <c r="W40" s="1" t="s">
-        <v>310</v>
+        <v>312</v>
       </c>
       <c r="X40" s="1" t="s">
-        <v>312</v>
+        <v>315</v>
       </c>
     </row>
     <row r="41" ht="15.75" customHeight="1">
       <c r="A41" s="1" t="s">
-        <v>313</v>
+        <v>316</v>
       </c>
       <c r="B41" s="1" t="s">
-        <v>314</v>
+        <v>317</v>
       </c>
       <c r="C41" s="1" t="s">
-        <v>315</v>
+        <v>318</v>
       </c>
       <c r="D41" s="1" t="s">
-        <v>251</v>
+        <v>255</v>
       </c>
       <c r="E41" s="1" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="F41" s="1" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="G41" s="1" t="s">
-        <v>251</v>
+        <v>255</v>
       </c>
       <c r="H41" s="1">
         <v>8200.0</v>
@@ -4038,48 +4133,51 @@
         <v>3.0</v>
       </c>
       <c r="L41" s="1" t="s">
-        <v>58</v>
+        <v>50</v>
       </c>
       <c r="M41" s="1" t="s">
-        <v>59</v>
+        <v>52</v>
+      </c>
+      <c r="O41" s="1" t="s">
+        <v>54</v>
       </c>
       <c r="P41" s="1" t="s">
-        <v>283</v>
+        <v>287</v>
       </c>
       <c r="S41" s="1" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="V41" s="1" t="s">
+        <v>319</v>
+      </c>
+      <c r="W41" s="1" t="s">
         <v>317</v>
       </c>
-      <c r="W41" s="1" t="s">
-        <v>316</v>
-      </c>
       <c r="X41" s="1" t="s">
-        <v>318</v>
+        <v>320</v>
       </c>
     </row>
     <row r="42" ht="15.75" customHeight="1">
       <c r="A42" s="1" t="s">
-        <v>319</v>
+        <v>321</v>
       </c>
       <c r="B42" s="1" t="s">
-        <v>320</v>
+        <v>322</v>
       </c>
       <c r="C42" s="1" t="s">
-        <v>321</v>
+        <v>323</v>
       </c>
       <c r="D42" s="1" t="s">
-        <v>251</v>
+        <v>255</v>
       </c>
       <c r="E42" s="1" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="F42" s="1" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="G42" s="1" t="s">
-        <v>251</v>
+        <v>255</v>
       </c>
       <c r="H42" s="1">
         <v>6900.0</v>
@@ -4094,48 +4192,51 @@
         <v>3.0</v>
       </c>
       <c r="L42" s="1" t="s">
-        <v>58</v>
+        <v>50</v>
       </c>
       <c r="M42" s="1" t="s">
-        <v>59</v>
+        <v>52</v>
+      </c>
+      <c r="O42" s="1" t="s">
+        <v>89</v>
       </c>
       <c r="P42" s="1" t="s">
-        <v>283</v>
+        <v>287</v>
       </c>
       <c r="S42" s="1" t="s">
         <v>322</v>
       </c>
       <c r="V42" s="1" t="s">
-        <v>323</v>
+        <v>324</v>
       </c>
       <c r="W42" s="1" t="s">
         <v>322</v>
       </c>
       <c r="X42" s="1" t="s">
-        <v>324</v>
+        <v>325</v>
       </c>
     </row>
     <row r="43" ht="15.75" customHeight="1">
       <c r="A43" s="1" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="B43" s="1" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="C43" s="1" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="D43" s="1" t="s">
-        <v>251</v>
+        <v>255</v>
       </c>
       <c r="E43" s="1" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="F43" s="1" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="G43" s="1" t="s">
-        <v>251</v>
+        <v>255</v>
       </c>
       <c r="H43" s="1">
         <v>13000.0</v>
@@ -4150,48 +4251,51 @@
         <v>3.0</v>
       </c>
       <c r="L43" s="1" t="s">
-        <v>58</v>
+        <v>50</v>
       </c>
       <c r="M43" s="1" t="s">
-        <v>59</v>
+        <v>52</v>
+      </c>
+      <c r="O43" s="1" t="s">
+        <v>54</v>
       </c>
       <c r="P43" s="1" t="s">
-        <v>283</v>
+        <v>287</v>
       </c>
       <c r="S43" s="1" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="V43" s="1" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="W43" s="1" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="X43" s="1" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
     </row>
     <row r="44" ht="15.75" customHeight="1">
       <c r="A44" s="1" t="s">
-        <v>330</v>
+        <v>331</v>
       </c>
       <c r="B44" s="1" t="s">
-        <v>331</v>
+        <v>332</v>
       </c>
       <c r="C44" s="1" t="s">
-        <v>332</v>
+        <v>333</v>
       </c>
       <c r="D44" s="1" t="s">
-        <v>251</v>
+        <v>255</v>
       </c>
       <c r="E44" s="1" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="F44" s="1" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="G44" s="1" t="s">
-        <v>251</v>
+        <v>255</v>
       </c>
       <c r="H44" s="1">
         <v>22000.0</v>
@@ -4206,54 +4310,57 @@
         <v>3.0</v>
       </c>
       <c r="L44" s="1" t="s">
-        <v>58</v>
+        <v>50</v>
       </c>
       <c r="M44" s="1" t="s">
-        <v>59</v>
+        <v>52</v>
+      </c>
+      <c r="O44" s="1" t="s">
+        <v>54</v>
       </c>
       <c r="P44" s="1" t="s">
-        <v>192</v>
+        <v>196</v>
       </c>
       <c r="Q44" s="1" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="R44" s="1" t="s">
+        <v>335</v>
+      </c>
+      <c r="S44" s="1" t="s">
+        <v>335</v>
+      </c>
+      <c r="V44" s="1" t="s">
+        <v>336</v>
+      </c>
+      <c r="W44" s="1" t="s">
         <v>334</v>
       </c>
-      <c r="S44" s="1" t="s">
-        <v>334</v>
-      </c>
-      <c r="V44" s="1" t="s">
-        <v>335</v>
-      </c>
-      <c r="W44" s="1" t="s">
-        <v>333</v>
-      </c>
       <c r="X44" s="1" t="s">
-        <v>336</v>
+        <v>337</v>
       </c>
     </row>
     <row r="45" ht="15.75" customHeight="1">
       <c r="A45" s="1" t="s">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="B45" s="1" t="s">
-        <v>338</v>
+        <v>339</v>
       </c>
       <c r="C45" s="1" t="s">
+        <v>340</v>
+      </c>
+      <c r="D45" s="1" t="s">
+        <v>218</v>
+      </c>
+      <c r="E45" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="F45" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="G45" s="1" t="s">
         <v>339</v>
-      </c>
-      <c r="D45" s="1" t="s">
-        <v>214</v>
-      </c>
-      <c r="E45" s="1" t="s">
-        <v>46</v>
-      </c>
-      <c r="F45" s="1" t="s">
-        <v>48</v>
-      </c>
-      <c r="G45" s="1" t="s">
-        <v>338</v>
       </c>
       <c r="H45" s="1">
         <v>30400.0</v>
@@ -4268,48 +4375,51 @@
         <v>3.0</v>
       </c>
       <c r="L45" s="1" t="s">
-        <v>58</v>
+        <v>50</v>
       </c>
       <c r="M45" s="1" t="s">
-        <v>59</v>
+        <v>52</v>
+      </c>
+      <c r="O45" s="1" t="s">
+        <v>54</v>
       </c>
       <c r="P45" s="1" t="s">
-        <v>192</v>
+        <v>196</v>
       </c>
       <c r="S45" s="1" t="s">
-        <v>338</v>
+        <v>339</v>
       </c>
       <c r="V45" s="1" t="s">
-        <v>340</v>
+        <v>341</v>
       </c>
       <c r="W45" s="1" t="s">
-        <v>338</v>
+        <v>339</v>
       </c>
       <c r="X45" s="1" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
     </row>
     <row r="46" ht="15.75" customHeight="1">
       <c r="A46" s="1" t="s">
-        <v>342</v>
+        <v>343</v>
       </c>
       <c r="B46" s="1" t="s">
-        <v>343</v>
+        <v>344</v>
       </c>
       <c r="C46" s="1" t="s">
+        <v>345</v>
+      </c>
+      <c r="D46" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="E46" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="F46" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="G46" s="1" t="s">
         <v>344</v>
-      </c>
-      <c r="D46" s="1" t="s">
-        <v>93</v>
-      </c>
-      <c r="E46" s="1" t="s">
-        <v>46</v>
-      </c>
-      <c r="F46" s="1" t="s">
-        <v>48</v>
-      </c>
-      <c r="G46" s="1" t="s">
-        <v>343</v>
       </c>
       <c r="H46" s="1">
         <v>32000.0</v>
@@ -4324,51 +4434,54 @@
         <v>0.0</v>
       </c>
       <c r="L46" s="1" t="s">
-        <v>58</v>
+        <v>50</v>
       </c>
       <c r="M46" s="1" t="s">
-        <v>59</v>
+        <v>52</v>
+      </c>
+      <c r="O46" s="1" t="s">
+        <v>54</v>
       </c>
       <c r="P46" s="1" t="s">
-        <v>192</v>
+        <v>196</v>
       </c>
       <c r="Q46" s="1" t="s">
-        <v>345</v>
+        <v>346</v>
       </c>
       <c r="S46" s="1" t="s">
-        <v>345</v>
+        <v>346</v>
       </c>
       <c r="V46" s="1" t="s">
+        <v>347</v>
+      </c>
+      <c r="W46" s="1" t="s">
         <v>346</v>
       </c>
-      <c r="W46" s="1" t="s">
-        <v>345</v>
-      </c>
       <c r="X46" s="1" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
     </row>
     <row r="47" ht="15.75" customHeight="1">
       <c r="A47" s="1" t="s">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="B47" s="1" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="C47" s="1" t="s">
-        <v>350</v>
+        <v>351</v>
       </c>
       <c r="D47" s="1" t="s">
-        <v>351</v>
+        <v>352</v>
       </c>
       <c r="E47" s="1" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F47" s="1" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="G47" s="1" t="s">
-        <v>351</v>
+        <v>352</v>
       </c>
       <c r="H47" s="1">
         <v>5900.0</v>
@@ -4383,48 +4496,51 @@
         <v>3.0</v>
       </c>
       <c r="L47" s="1" t="s">
-        <v>58</v>
+        <v>50</v>
       </c>
       <c r="M47" s="1" t="s">
-        <v>59</v>
+        <v>52</v>
+      </c>
+      <c r="O47" s="1" t="s">
+        <v>69</v>
       </c>
       <c r="P47" s="1" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="S47" s="1" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="V47" s="1" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="W47" s="1" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="X47" s="1" t="s">
-        <v>353</v>
+        <v>354</v>
       </c>
     </row>
     <row r="48" ht="15.75" customHeight="1">
       <c r="A48" s="1" t="s">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="B48" s="1" t="s">
-        <v>355</v>
+        <v>356</v>
       </c>
       <c r="C48" s="1" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="D48" s="1" t="s">
-        <v>200</v>
+        <v>204</v>
       </c>
       <c r="E48" s="1" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="F48" s="1" t="s">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="G48" s="1" t="s">
-        <v>200</v>
+        <v>204</v>
       </c>
       <c r="H48" s="1">
         <v>7800.0</v>
@@ -4439,48 +4555,51 @@
         <v>3.0</v>
       </c>
       <c r="L48" s="1" t="s">
-        <v>58</v>
+        <v>50</v>
       </c>
       <c r="M48" s="1" t="s">
-        <v>59</v>
+        <v>52</v>
+      </c>
+      <c r="O48" s="1" t="s">
+        <v>89</v>
       </c>
       <c r="P48" s="1" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="S48" s="1" t="s">
-        <v>355</v>
+        <v>356</v>
       </c>
       <c r="V48" s="1" t="s">
-        <v>357</v>
+        <v>358</v>
       </c>
       <c r="W48" s="1" t="s">
-        <v>355</v>
+        <v>356</v>
       </c>
       <c r="X48" s="1" t="s">
-        <v>358</v>
+        <v>359</v>
       </c>
     </row>
     <row r="49" ht="15.75" customHeight="1">
       <c r="A49" s="1" t="s">
-        <v>359</v>
+        <v>360</v>
       </c>
       <c r="B49" s="1" t="s">
-        <v>360</v>
+        <v>361</v>
       </c>
       <c r="C49" s="1" t="s">
-        <v>361</v>
+        <v>362</v>
       </c>
       <c r="D49" s="1" t="s">
-        <v>362</v>
+        <v>363</v>
       </c>
       <c r="E49" s="1" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="F49" s="1" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="G49" s="1" t="s">
-        <v>362</v>
+        <v>363</v>
       </c>
       <c r="H49" s="1">
         <v>14200.0</v>
@@ -4495,22 +4614,25 @@
         <v>3.0</v>
       </c>
       <c r="L49" s="1" t="s">
-        <v>58</v>
+        <v>50</v>
       </c>
       <c r="M49" s="1" t="s">
-        <v>59</v>
+        <v>52</v>
+      </c>
+      <c r="O49" s="1" t="s">
+        <v>54</v>
       </c>
       <c r="P49" s="1" t="s">
-        <v>283</v>
+        <v>287</v>
       </c>
       <c r="S49" s="1" t="s">
-        <v>363</v>
+        <v>361</v>
       </c>
       <c r="V49" s="1" t="s">
         <v>364</v>
       </c>
       <c r="W49" s="1" t="s">
-        <v>363</v>
+        <v>361</v>
       </c>
       <c r="X49" s="1" t="s">
         <v>365</v>
@@ -4527,16 +4649,16 @@
         <v>368</v>
       </c>
       <c r="D50" s="1" t="s">
-        <v>214</v>
+        <v>218</v>
       </c>
       <c r="E50" s="1" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="F50" s="1" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="G50" s="1" t="s">
-        <v>214</v>
+        <v>218</v>
       </c>
       <c r="H50" s="1">
         <v>13995.0</v>
@@ -4551,13 +4673,16 @@
         <v>3.0</v>
       </c>
       <c r="L50" s="1" t="s">
-        <v>58</v>
+        <v>50</v>
       </c>
       <c r="M50" s="1" t="s">
-        <v>59</v>
+        <v>52</v>
+      </c>
+      <c r="O50" s="1" t="s">
+        <v>54</v>
       </c>
       <c r="P50" s="1" t="s">
-        <v>283</v>
+        <v>287</v>
       </c>
       <c r="S50" s="1" t="s">
         <v>367</v>
@@ -4583,16 +4708,16 @@
         <v>373</v>
       </c>
       <c r="D51" s="1" t="s">
-        <v>362</v>
+        <v>363</v>
       </c>
       <c r="E51" s="1" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="F51" s="1" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="G51" s="1" t="s">
-        <v>362</v>
+        <v>363</v>
       </c>
       <c r="H51" s="1">
         <v>17000.0</v>
@@ -4607,13 +4732,16 @@
         <v>3.0</v>
       </c>
       <c r="L51" s="1" t="s">
-        <v>58</v>
+        <v>50</v>
       </c>
       <c r="M51" s="1" t="s">
-        <v>59</v>
+        <v>52</v>
+      </c>
+      <c r="O51" s="1" t="s">
+        <v>54</v>
       </c>
       <c r="P51" s="1" t="s">
-        <v>283</v>
+        <v>287</v>
       </c>
       <c r="S51" s="1" t="s">
         <v>372</v>
@@ -4639,16 +4767,16 @@
         <v>378</v>
       </c>
       <c r="D52" s="1" t="s">
-        <v>362</v>
+        <v>363</v>
       </c>
       <c r="E52" s="1" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F52" s="1" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="G52" s="1" t="s">
-        <v>362</v>
+        <v>363</v>
       </c>
       <c r="H52" s="1">
         <v>4700.0</v>
@@ -4663,13 +4791,16 @@
         <v>3.0</v>
       </c>
       <c r="L52" s="1" t="s">
-        <v>58</v>
+        <v>50</v>
       </c>
       <c r="M52" s="1" t="s">
-        <v>59</v>
+        <v>52</v>
+      </c>
+      <c r="O52" s="1" t="s">
+        <v>54</v>
       </c>
       <c r="P52" s="1" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="S52" s="1" t="s">
         <v>377</v>
@@ -4695,16 +4826,16 @@
         <v>383</v>
       </c>
       <c r="D53" s="1" t="s">
-        <v>214</v>
+        <v>218</v>
       </c>
       <c r="E53" s="1" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="F53" s="1" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="G53" s="1" t="s">
-        <v>214</v>
+        <v>218</v>
       </c>
       <c r="H53" s="1">
         <v>20200.0</v>
@@ -4719,13 +4850,16 @@
         <v>3.0</v>
       </c>
       <c r="L53" s="1" t="s">
-        <v>58</v>
+        <v>50</v>
       </c>
       <c r="M53" s="1" t="s">
-        <v>59</v>
+        <v>52</v>
+      </c>
+      <c r="O53" s="1" t="s">
+        <v>54</v>
       </c>
       <c r="P53" s="1" t="s">
-        <v>277</v>
+        <v>281</v>
       </c>
       <c r="S53" s="1" t="s">
         <v>382</v>
@@ -4754,10 +4888,10 @@
         <v>389</v>
       </c>
       <c r="E54" s="1" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="F54" s="1" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="G54" s="1" t="s">
         <v>389</v>
@@ -4775,13 +4909,16 @@
         <v>3.0</v>
       </c>
       <c r="L54" s="1" t="s">
-        <v>58</v>
+        <v>50</v>
       </c>
       <c r="M54" s="1" t="s">
-        <v>59</v>
+        <v>52</v>
+      </c>
+      <c r="O54" s="1" t="s">
+        <v>54</v>
       </c>
       <c r="P54" s="1" t="s">
-        <v>277</v>
+        <v>281</v>
       </c>
       <c r="S54" s="1" t="s">
         <v>387</v>
@@ -4810,10 +4947,10 @@
         <v>395</v>
       </c>
       <c r="E55" s="1" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="F55" s="1" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="G55" s="1" t="s">
         <v>395</v>
@@ -4831,13 +4968,16 @@
         <v>3.0</v>
       </c>
       <c r="L55" s="1" t="s">
-        <v>58</v>
+        <v>50</v>
       </c>
       <c r="M55" s="1" t="s">
-        <v>59</v>
+        <v>52</v>
+      </c>
+      <c r="O55" s="1" t="s">
+        <v>54</v>
       </c>
       <c r="P55" s="1" t="s">
-        <v>277</v>
+        <v>281</v>
       </c>
       <c r="S55" s="1" t="s">
         <v>393</v>
@@ -4866,10 +5006,10 @@
         <v>401</v>
       </c>
       <c r="E56" s="1" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="F56" s="1" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="G56" s="1" t="s">
         <v>399</v>
@@ -4887,10 +5027,13 @@
         <v>0.0</v>
       </c>
       <c r="L56" s="1" t="s">
-        <v>58</v>
+        <v>50</v>
       </c>
       <c r="M56" s="1" t="s">
-        <v>59</v>
+        <v>52</v>
+      </c>
+      <c r="O56" s="1" t="s">
+        <v>54</v>
       </c>
       <c r="P56" s="1" t="s">
         <v>402</v>
@@ -4925,16 +5068,16 @@
         <v>409</v>
       </c>
       <c r="D57" s="1" t="s">
-        <v>214</v>
+        <v>218</v>
       </c>
       <c r="E57" s="1" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="F57" s="1" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="G57" s="1" t="s">
-        <v>214</v>
+        <v>218</v>
       </c>
       <c r="H57" s="1">
         <v>13000.0</v>
@@ -4949,48 +5092,51 @@
         <v>3.0</v>
       </c>
       <c r="L57" s="1" t="s">
-        <v>58</v>
+        <v>50</v>
       </c>
       <c r="M57" s="1" t="s">
-        <v>59</v>
+        <v>52</v>
+      </c>
+      <c r="O57" s="1" t="s">
+        <v>54</v>
       </c>
       <c r="P57" s="1" t="s">
-        <v>283</v>
+        <v>287</v>
       </c>
       <c r="S57" s="1" t="s">
+        <v>408</v>
+      </c>
+      <c r="V57" s="1" t="s">
         <v>410</v>
       </c>
-      <c r="V57" s="1" t="s">
+      <c r="W57" s="1" t="s">
+        <v>408</v>
+      </c>
+      <c r="X57" s="1" t="s">
         <v>411</v>
-      </c>
-      <c r="W57" s="1" t="s">
-        <v>410</v>
-      </c>
-      <c r="X57" s="1" t="s">
-        <v>412</v>
       </c>
     </row>
     <row r="58" ht="15.75" customHeight="1">
       <c r="A58" s="1" t="s">
+        <v>412</v>
+      </c>
+      <c r="B58" s="1" t="s">
         <v>413</v>
       </c>
-      <c r="B58" s="1" t="s">
+      <c r="C58" s="1" t="s">
         <v>414</v>
       </c>
-      <c r="C58" s="1" t="s">
-        <v>415</v>
-      </c>
       <c r="D58" s="1" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="E58" s="1" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="F58" s="1" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="G58" s="1" t="s">
-        <v>414</v>
+        <v>413</v>
       </c>
       <c r="H58" s="1">
         <v>8500.0</v>
@@ -5005,48 +5151,51 @@
         <v>1.0</v>
       </c>
       <c r="L58" s="1" t="s">
-        <v>58</v>
+        <v>50</v>
       </c>
       <c r="M58" s="1" t="s">
-        <v>59</v>
+        <v>52</v>
+      </c>
+      <c r="O58" s="1" t="s">
+        <v>54</v>
       </c>
       <c r="P58" s="1" t="s">
-        <v>283</v>
+        <v>287</v>
       </c>
       <c r="S58" s="1" t="s">
-        <v>414</v>
+        <v>413</v>
       </c>
       <c r="V58" s="1" t="s">
+        <v>415</v>
+      </c>
+      <c r="W58" s="1" t="s">
+        <v>413</v>
+      </c>
+      <c r="X58" s="1" t="s">
         <v>416</v>
-      </c>
-      <c r="W58" s="1" t="s">
-        <v>414</v>
-      </c>
-      <c r="X58" s="1" t="s">
-        <v>417</v>
       </c>
     </row>
     <row r="59" ht="15.75" customHeight="1">
       <c r="A59" s="1" t="s">
+        <v>417</v>
+      </c>
+      <c r="B59" s="1" t="s">
         <v>418</v>
       </c>
-      <c r="B59" s="1" t="s">
+      <c r="C59" s="1" t="s">
         <v>419</v>
       </c>
-      <c r="C59" s="1" t="s">
+      <c r="D59" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="E59" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="F59" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="G59" s="1" t="s">
         <v>420</v>
-      </c>
-      <c r="D59" s="1" t="s">
-        <v>49</v>
-      </c>
-      <c r="E59" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="F59" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="G59" s="1" t="s">
-        <v>421</v>
       </c>
       <c r="H59" s="1">
         <v>7300.0</v>
@@ -5061,48 +5210,51 @@
         <v>1.0</v>
       </c>
       <c r="L59" s="1" t="s">
-        <v>58</v>
+        <v>50</v>
       </c>
       <c r="M59" s="1" t="s">
-        <v>59</v>
+        <v>52</v>
+      </c>
+      <c r="O59" s="1" t="s">
+        <v>89</v>
       </c>
       <c r="P59" s="1" t="s">
-        <v>283</v>
+        <v>287</v>
       </c>
       <c r="S59" s="1" t="s">
-        <v>419</v>
+        <v>418</v>
       </c>
       <c r="V59" s="1" t="s">
+        <v>421</v>
+      </c>
+      <c r="W59" s="1" t="s">
+        <v>418</v>
+      </c>
+      <c r="X59" s="1" t="s">
         <v>422</v>
-      </c>
-      <c r="W59" s="1" t="s">
-        <v>419</v>
-      </c>
-      <c r="X59" s="1" t="s">
-        <v>423</v>
       </c>
     </row>
     <row r="60" ht="15.75" customHeight="1">
       <c r="A60" s="1" t="s">
+        <v>423</v>
+      </c>
+      <c r="B60" s="1" t="s">
         <v>424</v>
       </c>
-      <c r="B60" s="1" t="s">
+      <c r="C60" s="1" t="s">
         <v>425</v>
       </c>
-      <c r="C60" s="1" t="s">
-        <v>426</v>
-      </c>
       <c r="D60" s="1" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="E60" s="1" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="F60" s="1" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="G60" s="1" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
       <c r="H60" s="1">
         <v>8200.0</v>
@@ -5117,48 +5269,51 @@
         <v>1.0</v>
       </c>
       <c r="L60" s="1" t="s">
-        <v>58</v>
+        <v>50</v>
       </c>
       <c r="M60" s="1" t="s">
-        <v>59</v>
+        <v>52</v>
+      </c>
+      <c r="O60" s="1" t="s">
+        <v>89</v>
       </c>
       <c r="P60" s="1" t="s">
-        <v>283</v>
+        <v>287</v>
       </c>
       <c r="S60" s="1" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
       <c r="V60" s="1" t="s">
+        <v>426</v>
+      </c>
+      <c r="W60" s="1" t="s">
+        <v>424</v>
+      </c>
+      <c r="X60" s="1" t="s">
         <v>427</v>
-      </c>
-      <c r="W60" s="1" t="s">
-        <v>425</v>
-      </c>
-      <c r="X60" s="1" t="s">
-        <v>428</v>
       </c>
     </row>
     <row r="61" ht="15.75" customHeight="1">
       <c r="A61" s="1" t="s">
+        <v>428</v>
+      </c>
+      <c r="B61" s="1" t="s">
         <v>429</v>
       </c>
-      <c r="B61" s="1" t="s">
+      <c r="C61" s="1" t="s">
         <v>430</v>
       </c>
-      <c r="C61" s="1" t="s">
-        <v>431</v>
-      </c>
       <c r="D61" s="1" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="E61" s="1" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="F61" s="1" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="G61" s="1" t="s">
-        <v>430</v>
+        <v>429</v>
       </c>
       <c r="H61" s="1">
         <v>17200.0</v>
@@ -5173,48 +5328,51 @@
         <v>1.0</v>
       </c>
       <c r="L61" s="1" t="s">
-        <v>58</v>
+        <v>50</v>
       </c>
       <c r="M61" s="1" t="s">
-        <v>59</v>
+        <v>52</v>
+      </c>
+      <c r="O61" s="1" t="s">
+        <v>89</v>
       </c>
       <c r="P61" s="1" t="s">
-        <v>283</v>
+        <v>287</v>
       </c>
       <c r="S61" s="1" t="s">
-        <v>430</v>
+        <v>429</v>
       </c>
       <c r="V61" s="1" t="s">
+        <v>431</v>
+      </c>
+      <c r="W61" s="1" t="s">
+        <v>429</v>
+      </c>
+      <c r="X61" s="1" t="s">
         <v>432</v>
-      </c>
-      <c r="W61" s="1" t="s">
-        <v>430</v>
-      </c>
-      <c r="X61" s="1" t="s">
-        <v>433</v>
       </c>
     </row>
     <row r="62" ht="15.75" customHeight="1">
       <c r="A62" s="1" t="s">
+        <v>433</v>
+      </c>
+      <c r="B62" s="1" t="s">
         <v>434</v>
       </c>
-      <c r="B62" s="1" t="s">
+      <c r="C62" s="1" t="s">
         <v>435</v>
       </c>
-      <c r="C62" s="1" t="s">
-        <v>436</v>
-      </c>
       <c r="D62" s="1" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="E62" s="1" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="F62" s="1" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="G62" s="1" t="s">
-        <v>435</v>
+        <v>434</v>
       </c>
       <c r="H62" s="1">
         <v>12200.0</v>
@@ -5229,48 +5387,51 @@
         <v>3.0</v>
       </c>
       <c r="L62" s="1" t="s">
-        <v>58</v>
+        <v>50</v>
       </c>
       <c r="M62" s="1" t="s">
-        <v>59</v>
+        <v>52</v>
+      </c>
+      <c r="O62" s="1" t="s">
+        <v>54</v>
       </c>
       <c r="P62" s="1" t="s">
-        <v>283</v>
+        <v>287</v>
       </c>
       <c r="S62" s="1" t="s">
-        <v>435</v>
+        <v>434</v>
       </c>
       <c r="V62" s="1" t="s">
+        <v>436</v>
+      </c>
+      <c r="W62" s="1" t="s">
+        <v>434</v>
+      </c>
+      <c r="X62" s="1" t="s">
         <v>437</v>
-      </c>
-      <c r="W62" s="1" t="s">
-        <v>435</v>
-      </c>
-      <c r="X62" s="1" t="s">
-        <v>438</v>
       </c>
     </row>
     <row r="63" ht="15.75" customHeight="1">
       <c r="A63" s="1" t="s">
+        <v>438</v>
+      </c>
+      <c r="B63" s="1" t="s">
         <v>439</v>
       </c>
-      <c r="B63" s="1" t="s">
+      <c r="C63" s="1" t="s">
         <v>440</v>
       </c>
-      <c r="C63" s="1" t="s">
-        <v>441</v>
-      </c>
       <c r="D63" s="1" t="s">
-        <v>214</v>
+        <v>218</v>
       </c>
       <c r="E63" s="1" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="F63" s="1" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="G63" s="1" t="s">
-        <v>214</v>
+        <v>218</v>
       </c>
       <c r="H63" s="1">
         <v>13100.0</v>
@@ -5285,48 +5446,51 @@
         <v>1.0</v>
       </c>
       <c r="L63" s="1" t="s">
-        <v>58</v>
+        <v>50</v>
       </c>
       <c r="M63" s="1" t="s">
-        <v>59</v>
+        <v>52</v>
+      </c>
+      <c r="O63" s="1" t="s">
+        <v>54</v>
       </c>
       <c r="P63" s="1" t="s">
-        <v>283</v>
+        <v>287</v>
       </c>
       <c r="S63" s="1" t="s">
-        <v>440</v>
+        <v>439</v>
       </c>
       <c r="V63" s="1" t="s">
+        <v>441</v>
+      </c>
+      <c r="W63" s="1" t="s">
+        <v>439</v>
+      </c>
+      <c r="X63" s="1" t="s">
         <v>442</v>
-      </c>
-      <c r="W63" s="1" t="s">
-        <v>440</v>
-      </c>
-      <c r="X63" s="1" t="s">
-        <v>443</v>
       </c>
     </row>
     <row r="64" ht="15.75" customHeight="1">
       <c r="A64" s="1" t="s">
+        <v>443</v>
+      </c>
+      <c r="B64" s="1" t="s">
         <v>444</v>
       </c>
-      <c r="B64" s="1" t="s">
+      <c r="C64" s="1" t="s">
         <v>445</v>
       </c>
-      <c r="C64" s="1" t="s">
-        <v>446</v>
-      </c>
       <c r="D64" s="1" t="s">
-        <v>362</v>
+        <v>363</v>
       </c>
       <c r="E64" s="1" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="F64" s="1" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="G64" s="1" t="s">
-        <v>362</v>
+        <v>363</v>
       </c>
       <c r="H64" s="1">
         <v>12500.0</v>
@@ -5341,48 +5505,51 @@
         <v>1.0</v>
       </c>
       <c r="L64" s="1" t="s">
-        <v>58</v>
+        <v>50</v>
       </c>
       <c r="M64" s="1" t="s">
-        <v>59</v>
+        <v>52</v>
+      </c>
+      <c r="O64" s="1" t="s">
+        <v>54</v>
       </c>
       <c r="P64" s="1" t="s">
-        <v>283</v>
+        <v>287</v>
       </c>
       <c r="S64" s="1" t="s">
-        <v>445</v>
+        <v>444</v>
       </c>
       <c r="V64" s="1" t="s">
+        <v>446</v>
+      </c>
+      <c r="W64" s="1" t="s">
+        <v>444</v>
+      </c>
+      <c r="X64" s="1" t="s">
         <v>447</v>
-      </c>
-      <c r="W64" s="1" t="s">
-        <v>445</v>
-      </c>
-      <c r="X64" s="1" t="s">
-        <v>448</v>
       </c>
     </row>
     <row r="65" ht="15.75" customHeight="1">
       <c r="A65" s="1" t="s">
+        <v>448</v>
+      </c>
+      <c r="B65" s="1" t="s">
         <v>449</v>
       </c>
-      <c r="B65" s="1" t="s">
+      <c r="C65" s="1" t="s">
         <v>450</v>
-      </c>
-      <c r="C65" s="1" t="s">
-        <v>451</v>
       </c>
       <c r="D65" s="1" t="s">
         <v>401</v>
       </c>
       <c r="E65" s="1" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="F65" s="1" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="G65" s="1" t="s">
-        <v>450</v>
+        <v>449</v>
       </c>
       <c r="H65" s="1">
         <v>73000.0</v>
@@ -5397,10 +5564,13 @@
         <v>0.0</v>
       </c>
       <c r="L65" s="1" t="s">
-        <v>58</v>
+        <v>50</v>
       </c>
       <c r="M65" s="1" t="s">
-        <v>59</v>
+        <v>52</v>
+      </c>
+      <c r="O65" s="1" t="s">
+        <v>54</v>
       </c>
       <c r="P65" s="1" t="s">
         <v>402</v>
@@ -5415,74 +5585,78 @@
         <v>404</v>
       </c>
       <c r="V65" s="1" t="s">
-        <v>452</v>
+        <v>451</v>
       </c>
       <c r="W65" s="1" t="s">
         <v>403</v>
       </c>
       <c r="X65" s="1" t="s">
-        <v>453</v>
+        <v>452</v>
       </c>
     </row>
     <row r="66" ht="15.75" customHeight="1">
-      <c r="A66" s="2" t="s">
+      <c r="A66" s="1" t="s">
+        <v>453</v>
+      </c>
+      <c r="B66" s="1" t="s">
         <v>454</v>
       </c>
-      <c r="B66" s="2" t="s">
+      <c r="C66" s="1" t="s">
         <v>455</v>
       </c>
-      <c r="C66" s="2" t="s">
+      <c r="D66" s="1" t="s">
+        <v>195</v>
+      </c>
+      <c r="E66" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="F66" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="G66" s="1" t="s">
+        <v>195</v>
+      </c>
+      <c r="H66" s="1">
+        <v>30000.0</v>
+      </c>
+      <c r="I66" s="1">
+        <v>25000.0</v>
+      </c>
+      <c r="J66" s="1">
+        <v>16.67</v>
+      </c>
+      <c r="K66" s="1">
+        <v>5.0</v>
+      </c>
+      <c r="L66" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="M66" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="O66" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="P66" s="1" t="s">
         <v>456</v>
       </c>
-      <c r="D66" s="2" t="s">
-        <v>191</v>
-      </c>
-      <c r="E66" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="F66" s="1" t="s">
-        <v>31</v>
-      </c>
-      <c r="G66" s="2" t="s">
-        <v>191</v>
-      </c>
-      <c r="H66" s="2">
-        <v>30000.0</v>
-      </c>
-      <c r="I66" s="2">
-        <v>25000.0</v>
-      </c>
-      <c r="K66" s="2">
-        <v>5.0</v>
-      </c>
-      <c r="L66" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="M66" s="1" t="s">
-        <v>59</v>
-      </c>
-      <c r="P66" s="2" t="s">
+      <c r="R66" s="1" t="s">
         <v>457</v>
       </c>
-      <c r="R66" s="3" t="s">
+      <c r="S66" s="1" t="s">
+        <v>457</v>
+      </c>
+      <c r="V66" s="1" t="s">
         <v>458</v>
       </c>
-      <c r="S66" s="2" t="s">
-        <v>458</v>
-      </c>
-      <c r="V66" s="2" t="s">
+      <c r="W66" s="1" t="s">
+        <v>457</v>
+      </c>
+      <c r="X66" s="1" t="s">
         <v>459</v>
       </c>
-      <c r="W66" s="2" t="s">
-        <v>458</v>
-      </c>
-      <c r="X66" s="2" t="s">
-        <v>460</v>
-      </c>
     </row>
-    <row r="67" ht="15.75" customHeight="1">
-      <c r="R67" s="4"/>
-    </row>
+    <row r="67" ht="15.75" customHeight="1"/>
     <row r="68" ht="15.75" customHeight="1"/>
     <row r="69" ht="15.75" customHeight="1"/>
     <row r="70" ht="15.75" customHeight="1"/>
@@ -6446,7 +6620,7 @@
         <v>4</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F1" s="1" t="s">
         <v>7</v>
@@ -6454,122 +6628,122 @@
     </row>
     <row r="2">
       <c r="A2" s="1" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="E3" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="F3" s="1" t="s">
         <v>27</v>
-      </c>
-      <c r="F3" s="1" t="s">
-        <v>25</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="1" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="F4" s="1" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="1" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>40</v>
+        <v>44</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>42</v>
+        <v>46</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="F5" s="1" t="s">
-        <v>42</v>
+        <v>46</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="1" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="F6" s="1" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="1" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>54</v>
+        <v>59</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>55</v>
+        <v>61</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>56</v>
+        <v>63</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>57</v>
+        <v>65</v>
       </c>
       <c r="F7" s="1" t="s">
-        <v>56</v>
+        <v>63</v>
       </c>
     </row>
     <row r="21" ht="15.75" customHeight="1"/>

</xml_diff>

<commit_message>
Branch: NEXT-PRE-DEVELOPMENT - feat: preserve existing SEO and metadata when importing products from Excel
</commit_message>
<xml_diff>
--- a/store_inventory_template.xlsx
+++ b/store_inventory_template.xlsx
@@ -398,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:K52"/>
+  <dimension ref="A1:L52"/>
   <cols>
     <col min="1" max="1" width="14.83203125" customWidth="1"/>
     <col min="2" max="2" width="35.83203125" customWidth="1"/>
@@ -410,7 +410,8 @@
     <col min="8" max="8" width="12.83203125" customWidth="1"/>
     <col min="9" max="9" width="16.83203125" customWidth="1"/>
     <col min="10" max="10" width="65.83203125" customWidth="1"/>
-    <col min="11" max="11" width="50.83203125" customWidth="1"/>
+    <col min="11" max="11" width="80.83203125" customWidth="1"/>
+    <col min="12" max="12" width="50.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -445,6 +446,9 @@
         <v>description</v>
       </c>
       <c r="K1" t="str">
+        <v>specifications</v>
+      </c>
+      <c r="L1" t="str">
         <v>images</v>
       </c>
     </row>
@@ -480,6 +484,9 @@
         <v>Durable and stylish adult cycle engineered with High-Tensile Carbon Steel Frame, High-Performance V-Brake System, and sleek geometry for daily commutes and fitness rides.</v>
       </c>
       <c r="K2" t="str">
+        <v>Wheel Size: 26 Inches | Frame Material: High-Tensile Carbon Steel Frame | Brake System: High-Performance V-Brake System | Gears / Speed: Single Speed Direct Drive | Front Suspension: Rigid Aerodynamic Steel Fork | Target Age Group: 15+ Years | Ideal Location: Urban Roads, Fitness Trails &amp; City Commuting</v>
+      </c>
+      <c r="L2" t="str">
         <v>/images/products/prod_001_1_1cBHXAZIQpKTodzPqbos1Ngp1sV-MFDwC.jpg,/images/products/prod_001_2_1Iv7MRj7lY8BSTD19GLEGM0ZcK6zuQYd1.jpg</v>
       </c>
     </row>
@@ -515,6 +522,9 @@
         <v>Sturdy and safe kids cycle designed for young riders (8-12 Years). Equipped with anti-skid tires, full chain guard, and ergonomic safety grips.</v>
       </c>
       <c r="K3" t="str">
+        <v>Wheel Size: 20 Inches | Frame Material: High-Tensile Carbon Steel Frame | Brake System: Calibrated Caliper Brakes with Child-Safe Levers | Gears / Speed: Single Speed Direct Drive | Front Suspension: Rigid Aerodynamic Steel Fork | Target Age Group: 8-12 Years | Ideal Location: Urban Roads, Fitness Trails &amp; City Commuting</v>
+      </c>
+      <c r="L3" t="str">
         <v>/images/products/prod_002_1_1UMFTn5JP9w2FFi4KL6l-8diVc5gUkx-Z.jpg</v>
       </c>
     </row>
@@ -550,6 +560,9 @@
         <v>Durable and stylish adult cycle engineered with High-Tensile Carbon Steel Frame, Dual Mechanical Disc Brakes (Front &amp; Rear), and sleek geometry for daily commutes and fitness rides.</v>
       </c>
       <c r="K4" t="str">
+        <v>Wheel Size: 24 Inches | Frame Material: High-Tensile Carbon Steel Frame | Brake System: Dual Mechanical Disc Brakes (Front &amp; Rear) | Gears / Speed: Single Speed Direct Drive | Front Suspension: Front Telescopic Suspension Fork | Target Age Group: 12-15 Years | Ideal Location: Urban Roads, Fitness Trails &amp; City Commuting</v>
+      </c>
+      <c r="L4" t="str">
         <v>/images/products/prod_005_1.jpg</v>
       </c>
     </row>
@@ -585,6 +598,9 @@
         <v>Durable and stylish adult cycle engineered with High-Tensile Carbon Steel Frame, Dual Mechanical Disc Brakes (Front &amp; Rear), and sleek geometry for daily commutes and fitness rides.</v>
       </c>
       <c r="K5" t="str">
+        <v>Wheel Size: 26 Inches | Frame Material: High-Tensile Carbon Steel Frame | Brake System: Dual Mechanical Disc Brakes (Front &amp; Rear) | Gears / Speed: Single Speed Direct Drive | Front Suspension: Front Telescopic Suspension Fork | Target Age Group: 15+ Years | Ideal Location: Urban Roads, Fitness Trails &amp; City Commuting</v>
+      </c>
+      <c r="L5" t="str">
         <v>/images/products/prod_006_1.jpg</v>
       </c>
     </row>
@@ -620,6 +636,9 @@
         <v>Elegant and comfortable girls cycle featuring low step-through frame, comfortable upright geometry, rear carrier, and smooth brake controls.</v>
       </c>
       <c r="K6" t="str">
+        <v>Wheel Size: 26 Inches | Frame Material: High-Tensile Carbon Steel Frame | Brake System: Front &amp; Rear Mechanical Power Brakes | Gears / Speed: Single Speed Direct Drive | Front Suspension: Rigid Aerodynamic Steel Fork | Target Age Group: 15+ Years | Ideal Location: Urban Roads, Fitness Trails &amp; City Commuting</v>
+      </c>
+      <c r="L6" t="str">
         <v>/images/products/prod_009_1.jpg</v>
       </c>
     </row>
@@ -655,6 +674,9 @@
         <v>Sturdy and safe kids cycle designed for young riders (8-12 Years). Equipped with anti-skid tires, full chain guard, and ergonomic safety grips.</v>
       </c>
       <c r="K7" t="str">
+        <v>Wheel Size: 20 Inches | Frame Material: High-Tensile Carbon Steel Frame | Brake System: Calibrated Caliper Brakes with Child-Safe Levers | Gears / Speed: Single Speed Direct Drive | Front Suspension: Rigid Aerodynamic Steel Fork | Target Age Group: 8-12 Years | Ideal Location: Urban Roads, Fitness Trails &amp; City Commuting</v>
+      </c>
+      <c r="L7" t="str">
         <v>/images/products/prod_011_1.jpg,/images/products/prod_011_2.jpg,/images/products/prod_011_3_1mab42s_Mf84sxHNRZbtB6q6yn-2m0tMB.jpg</v>
       </c>
     </row>
@@ -690,6 +712,9 @@
         <v>Elegant and comfortable girls cycle featuring low step-through frame, comfortable upright geometry, rear carrier, and smooth brake controls.</v>
       </c>
       <c r="K8" t="str">
+        <v>Wheel Size: 24 Inches | Frame Material: High-Tensile Carbon Steel Frame | Brake System: Front &amp; Rear Mechanical Power Brakes | Gears / Speed: Single Speed Direct Drive | Front Suspension: Rigid Aerodynamic Steel Fork | Target Age Group: 12-15 Years | Ideal Location: Urban Roads, Fitness Trails &amp; City Commuting</v>
+      </c>
+      <c r="L8" t="str">
         <v>/images/products/prod_012_1.jpg,/images/products/prod_012_2.jpg,/images/products/prod_012_3.jpg</v>
       </c>
     </row>
@@ -725,6 +750,9 @@
         <v>Avon Yama 26T FAT is a rugged fat-tire bicycle featuring extra-wide 4.0" all-terrain tires, heavy-duty suspension, and 21-speed gears for ultimate traction and off-road dominance.</v>
       </c>
       <c r="K9" t="str">
+        <v>Wheel Size: 26 Inches | Frame Material: High-Tensile Carbon Steel Frame | Brake System: Front &amp; Rear Mechanical Power Brakes | Gears / Speed: Multi-Speed Gear System | Front Suspension: Rigid Aerodynamic Steel Fork | Target Age Group: 15+ Years | Ideal Location: Urban Roads, Fitness Trails &amp; City Commuting | Tire Dimensions: 26 x 4.0 Inch Ultra-Wide All-Terrain Tread</v>
+      </c>
+      <c r="L9" t="str">
         <v>/images/products/prod_013_1.jpg,/images/products/prod_013_2.jpg,/images/products/prod_013_3.jpg</v>
       </c>
     </row>
@@ -760,6 +788,9 @@
         <v>Sturdy and safe kids cycle designed for young riders (2-5 Years). Equipped with anti-skid tires, full chain guard, and ergonomic safety grips.</v>
       </c>
       <c r="K10" t="str">
+        <v>Wheel Size: 12 Inches | Frame Material: High-Tensile Carbon Steel Frame | Brake System: Calibrated Caliper Brakes with Child-Safe Levers | Gears / Speed: Single Speed Direct Drive | Front Suspension: Rigid Aerodynamic Steel Fork | Target Age Group: 2-5 Years | Ideal Location: Urban Roads, Fitness Trails &amp; City Commuting</v>
+      </c>
+      <c r="L10" t="str">
         <v>/images/products/prod_014_1.jpg</v>
       </c>
     </row>
@@ -795,6 +826,9 @@
         <v>Sturdy and safe kids cycle designed for young riders (2-5 Years). Equipped with anti-skid tires, full chain guard, and ergonomic safety grips.</v>
       </c>
       <c r="K11" t="str">
+        <v>Wheel Size: 14 Inches | Frame Material: High-Tensile Carbon Steel Frame | Brake System: Calibrated Caliper Brakes with Child-Safe Levers | Gears / Speed: Single Speed Direct Drive | Front Suspension: Rigid Aerodynamic Steel Fork | Target Age Group: 2-5 Years | Ideal Location: Urban Roads, Fitness Trails &amp; City Commuting</v>
+      </c>
+      <c r="L11" t="str">
         <v>/images/products/prod_015_1.jpg</v>
       </c>
     </row>
@@ -830,6 +864,9 @@
         <v>Sturdy and safe kids cycle designed for young riders (5-8 Years). Equipped with anti-skid tires, full chain guard, and ergonomic safety grips.</v>
       </c>
       <c r="K12" t="str">
+        <v>Wheel Size: 16 Inches | Frame Material: High-Tensile Carbon Steel Frame | Brake System: Calibrated Caliper Brakes with Child-Safe Levers | Gears / Speed: Single Speed Direct Drive | Front Suspension: Rigid Aerodynamic Steel Fork | Target Age Group: 5-8 Years | Ideal Location: Urban Roads, Fitness Trails &amp; City Commuting</v>
+      </c>
+      <c r="L12" t="str">
         <v>/images/products/prod_016_1.jpg</v>
       </c>
     </row>
@@ -865,6 +902,9 @@
         <v>Sturdy and safe kids cycle designed for young riders (8-12 Years). Equipped with anti-skid tires, full chain guard, and ergonomic safety grips.</v>
       </c>
       <c r="K13" t="str">
+        <v>Wheel Size: 20 Inches | Frame Material: High-Tensile Carbon Steel Frame | Brake System: Calibrated Caliper Brakes with Child-Safe Levers | Gears / Speed: Single Speed Direct Drive | Front Suspension: Rigid Aerodynamic Steel Fork | Target Age Group: 8-12 Years | Ideal Location: Urban Roads, Fitness Trails &amp; City Commuting</v>
+      </c>
+      <c r="L13" t="str">
         <v>/images/products/prod_017_1.jpg</v>
       </c>
     </row>
@@ -900,6 +940,9 @@
         <v>Sturdy and safe kids cycle designed for young riders (8-12 Years). Equipped with anti-skid tires, full chain guard, and ergonomic safety grips.</v>
       </c>
       <c r="K14" t="str">
+        <v>Wheel Size: 20 Inches | Frame Material: High-Tensile Carbon Steel Frame | Brake System: Caliper Brakes with Soft-Grip Rubber Pads | Gears / Speed: Single Speed Direct Drive | Front Suspension: Rigid Aerodynamic Steel Fork | Target Age Group: 8-12 Years | Ideal Location: Urban Roads, Fitness Trails &amp; City Commuting</v>
+      </c>
+      <c r="L14" t="str">
         <v>/images/products/prod_018_1.jpg</v>
       </c>
     </row>
@@ -935,6 +978,9 @@
         <v>Durable and stylish adult cycle engineered with High-Tensile Carbon Steel Frame, Dual Mechanical Disc Brakes (Front &amp; Rear), and sleek geometry for daily commutes and fitness rides.</v>
       </c>
       <c r="K15" t="str">
+        <v>Wheel Size: 26 Inches | Frame Material: High-Tensile Carbon Steel Frame | Brake System: Dual Mechanical Disc Brakes (Front &amp; Rear) | Gears / Speed: Single Speed Direct Drive | Front Suspension: Rigid Aerodynamic Steel Fork | Target Age Group: 15+ Years | Ideal Location: Urban Roads, Fitness Trails &amp; City Commuting</v>
+      </c>
+      <c r="L15" t="str">
         <v>/images/products/prod_019_1.jpg</v>
       </c>
     </row>
@@ -970,6 +1016,9 @@
         <v>Durable and stylish adult cycle engineered with High-Tensile Carbon Steel Frame, Dual Mechanical Disc Brakes (Front &amp; Rear), and sleek geometry for daily commutes and fitness rides.</v>
       </c>
       <c r="K16" t="str">
+        <v>Wheel Size: 24 Inches | Frame Material: High-Tensile Carbon Steel Frame | Brake System: Dual Mechanical Disc Brakes (Front &amp; Rear) | Gears / Speed: Single Speed Direct Drive | Front Suspension: Front Telescopic Suspension Fork | Target Age Group: 12-15 Years | Ideal Location: Urban Roads, Fitness Trails &amp; City Commuting</v>
+      </c>
+      <c r="L16" t="str">
         <v>/images/products/prod_020_1.jpg</v>
       </c>
     </row>
@@ -1005,6 +1054,9 @@
         <v>Montra Hypno PRO 27T EC is an advanced electric bicycle powered by a high-torque BLDC hub motor and removable lithium battery, designed for long-range commutes across Tirunelveli.</v>
       </c>
       <c r="K17" t="str">
+        <v>Wheel Size: 27.5 Inches | Frame Material: Lightweight Aircraft-Grade Alloy Frame | Brake System: Front &amp; Rear Mechanical Power Brakes | Gears / Speed: Single Speed Direct Drive | Front Suspension: Rigid Aerodynamic Steel Fork | Target Age Group: 15+ Years | Ideal Location: Urban Roads, Fitness Trails &amp; City Commuting | Motor Type: 36V 250W High-Torque Rear Hub BLDC Motor | Battery Unit: Removable 36V Lithium-Ion LFP Battery Pack | Riding Modes: Pedal Assist (PAS) &amp; Pure Throttle Mode | Top Speed: Up to 25 km/h</v>
+      </c>
+      <c r="L17" t="str">
         <v>/images/products/prod_021_1.jpg,/images/products/prod_021_2.jpg</v>
       </c>
     </row>
@@ -1040,6 +1092,9 @@
         <v>BSA Viona 26T is an advanced electric bicycle powered by a high-torque BLDC hub motor and removable lithium battery, designed for long-range commutes across Tirunelveli.</v>
       </c>
       <c r="K18" t="str">
+        <v>Wheel Size: 26 Inches | Frame Material: High-Tensile Carbon Steel Frame | Brake System: Front &amp; Rear Mechanical Power Brakes | Gears / Speed: Single Speed Direct Drive | Front Suspension: Rigid Aerodynamic Steel Fork | Target Age Group: 15+ Years | Ideal Location: Urban Roads, Fitness Trails &amp; City Commuting | Motor Type: 36V 250W High-Torque Rear Hub BLDC Motor | Battery Unit: Removable 36V Lithium-Ion LFP Battery Pack | Riding Modes: Pedal Assist (PAS) &amp; Pure Throttle Mode | Top Speed: Up to 25 km/h</v>
+      </c>
+      <c r="L18" t="str">
         <v>/images/products/prod_022_1.jpg,/images/products/prod_022_2.jpg,/images/products/prod_022_3.jpg</v>
       </c>
     </row>
@@ -1075,6 +1130,9 @@
         <v>Durable and stylish adult cycle engineered with Lightweight Aircraft-Grade Alloy Frame, Dual Mechanical Disc Brakes (Front &amp; Rear), and sleek geometry for daily commutes and fitness rides.</v>
       </c>
       <c r="K19" t="str">
+        <v>Wheel Size: 29 Inches | Frame Material: Lightweight Aircraft-Grade Alloy Frame | Brake System: Dual Mechanical Disc Brakes (Front &amp; Rear) | Gears / Speed: Single Speed Direct Drive | Front Suspension: Rigid Aerodynamic Steel Fork | Target Age Group: 15+ Years | Ideal Location: Urban Roads, Fitness Trails &amp; City Commuting</v>
+      </c>
+      <c r="L19" t="str">
         <v>/images/products/prod_024_1.jpg,/images/products/prod_024_2.jpg,/images/products/prod_024_3.jpg</v>
       </c>
     </row>
@@ -1110,6 +1168,9 @@
         <v>Maeve 26T EC is an advanced electric bicycle powered by a high-torque BLDC hub motor and removable lithium battery, designed for long-range commutes across Tirunelveli.</v>
       </c>
       <c r="K20" t="str">
+        <v>Wheel Size: 26 Inches | Frame Material: High-Tensile Carbon Steel Frame | Brake System: Front &amp; Rear Mechanical Power Brakes | Gears / Speed: Single Speed Direct Drive | Front Suspension: Rigid Aerodynamic Steel Fork | Target Age Group: 15+ Years | Ideal Location: Urban Roads, Fitness Trails &amp; City Commuting | Motor Type: 36V 250W High-Torque Rear Hub BLDC Motor | Battery Unit: Removable 36V Lithium-Ion LFP Battery Pack | Riding Modes: Pedal Assist (PAS) &amp; Pure Throttle Mode | Top Speed: Up to 25 km/h</v>
+      </c>
+      <c r="L20" t="str">
         <v>/images/products/prod_025_1.jpg</v>
       </c>
     </row>
@@ -1145,6 +1206,9 @@
         <v>High-performance geared cycle built with 21-Speed Gear System (Shimano / Microshift), Dual Mechanical Disc Brakes (Front &amp; Rear), and a rigid High-Tensile Carbon Steel Frame for fast city and trail riding.</v>
       </c>
       <c r="K21" t="str">
+        <v>Wheel Size: 29 Inches | Frame Material: High-Tensile Carbon Steel Frame | Brake System: Dual Mechanical Disc Brakes (Front &amp; Rear) | Gears / Speed: 21-Speed Gear System (Shimano / Microshift) | Front Suspension: Front Telescopic Suspension Fork | Target Age Group: 15+ Years | Ideal Location: Urban Roads, Fitness Trails &amp; City Commuting</v>
+      </c>
+      <c r="L21" t="str">
         <v>/images/products/prod_027_1.jpg</v>
       </c>
     </row>
@@ -1180,6 +1244,9 @@
         <v>Hercules Brute 27T FSDD EC is an advanced electric bicycle powered by a high-torque BLDC hub motor and removable lithium battery, designed for long-range commutes across Tirunelveli.</v>
       </c>
       <c r="K22" t="str">
+        <v>Wheel Size: 27.5 Inches | Frame Material: High-Tensile Carbon Steel Frame | Brake System: Dual Mechanical Disc Brakes (Front &amp; Rear) | Gears / Speed: Single Speed Direct Drive | Front Suspension: Front Telescopic Suspension Fork | Target Age Group: 15+ Years | Ideal Location: Urban Roads, Fitness Trails &amp; City Commuting | Motor Type: 36V 250W High-Torque Rear Hub BLDC Motor | Battery Unit: Removable 36V Lithium-Ion LFP Battery Pack | Riding Modes: Pedal Assist (PAS) &amp; Pure Throttle Mode | Top Speed: Up to 25 km/h</v>
+      </c>
+      <c r="L22" t="str">
         <v>/images/products/prod_029_1.jpg</v>
       </c>
     </row>
@@ -1215,6 +1282,9 @@
         <v>Sturdy and safe kids cycle designed for young riders (8-12 Years). Equipped with anti-skid tires, full chain guard, and ergonomic safety grips.</v>
       </c>
       <c r="K23" t="str">
+        <v>Wheel Size: 20 Inches | Frame Material: High-Tensile Carbon Steel Frame | Brake System: Calibrated Caliper Brakes with Child-Safe Levers | Gears / Speed: Single Speed Direct Drive | Front Suspension: Rigid Aerodynamic Steel Fork | Target Age Group: 8-12 Years | Ideal Location: Urban Roads, Fitness Trails &amp; City Commuting</v>
+      </c>
+      <c r="L23" t="str">
         <v>/images/products/prod_030_1.jpg</v>
       </c>
     </row>
@@ -1250,6 +1320,9 @@
         <v>Sturdy and safe kids cycle designed for young riders (8-12 Years). Equipped with anti-skid tires, full chain guard, and ergonomic safety grips.</v>
       </c>
       <c r="K24" t="str">
+        <v>Wheel Size: 20 Inches | Frame Material: High-Tensile Carbon Steel Frame | Brake System: Calibrated Caliper Brakes with Child-Safe Levers | Gears / Speed: Single Speed Direct Drive | Front Suspension: Rigid Aerodynamic Steel Fork | Target Age Group: 8-12 Years | Ideal Location: Urban Roads, Fitness Trails &amp; City Commuting</v>
+      </c>
+      <c r="L24" t="str">
         <v>/images/products/prod_031_1.jpg</v>
       </c>
     </row>
@@ -1285,6 +1358,9 @@
         <v>Hercules Hardstyle PRO 27T EC is an advanced electric bicycle powered by a high-torque BLDC hub motor and removable lithium battery, designed for long-range commutes across Tirunelveli.</v>
       </c>
       <c r="K25" t="str">
+        <v>Wheel Size: 27.5 Inches | Frame Material: High-Tensile Carbon Steel Frame | Brake System: Front &amp; Rear Mechanical Power Brakes | Gears / Speed: Single Speed Direct Drive | Front Suspension: Rigid Aerodynamic Steel Fork | Target Age Group: 15+ Years | Ideal Location: Urban Roads, Fitness Trails &amp; City Commuting | Motor Type: 36V 250W High-Torque Rear Hub BLDC Motor | Battery Unit: Removable 36V Lithium-Ion LFP Battery Pack | Riding Modes: Pedal Assist (PAS) &amp; Pure Throttle Mode | Top Speed: Up to 25 km/h</v>
+      </c>
+      <c r="L25" t="str">
         <v>/images/products/prod_032_1.jpg</v>
       </c>
     </row>
@@ -1320,6 +1396,9 @@
         <v>High-performance geared cycle built with 21-Speed Gear System (Shimano / Microshift), Dual Mechanical Disc Brakes (Front &amp; Rear), and a rigid High-Tensile Carbon Steel Frame for fast city and trail riding.</v>
       </c>
       <c r="K26" t="str">
+        <v>Wheel Size: 27.5 Inches | Frame Material: High-Tensile Carbon Steel Frame | Brake System: Dual Mechanical Disc Brakes (Front &amp; Rear) | Gears / Speed: 21-Speed Gear System (Shimano / Microshift) | Front Suspension: Rigid Aerodynamic Steel Fork | Target Age Group: 15+ Years | Ideal Location: Urban Roads, Fitness Trails &amp; City Commuting</v>
+      </c>
+      <c r="L26" t="str">
         <v>/images/products/prod_033_1.jpg</v>
       </c>
     </row>
@@ -1355,6 +1434,9 @@
         <v>Durable and stylish adult cycle engineered with High-Tensile Carbon Steel Frame, High-Performance V-Brake System, and sleek geometry for daily commutes and fitness rides.</v>
       </c>
       <c r="K27" t="str">
+        <v>Wheel Size: 26 Inches | Frame Material: High-Tensile Carbon Steel Frame | Brake System: High-Performance V-Brake System | Gears / Speed: Single Speed Direct Drive | Front Suspension: Rigid Aerodynamic Steel Fork | Target Age Group: 15+ Years | Ideal Location: Urban Roads, Fitness Trails &amp; City Commuting</v>
+      </c>
+      <c r="L27" t="str">
         <v>/images/products/prod_034_1.jpg</v>
       </c>
     </row>
@@ -1390,6 +1472,9 @@
         <v>Sturdy and safe kids cycle designed for young riders (2-5 Years). Equipped with anti-skid tires, full chain guard, and ergonomic safety grips.</v>
       </c>
       <c r="K28" t="str">
+        <v>Wheel Size: 14 Inches | Frame Material: High-Tensile Carbon Steel Frame | Brake System: Calibrated Caliper Brakes with Child-Safe Levers | Gears / Speed: Single Speed Direct Drive | Front Suspension: Rigid Aerodynamic Steel Fork | Target Age Group: 2-5 Years | Ideal Location: Urban Roads, Fitness Trails &amp; City Commuting</v>
+      </c>
+      <c r="L28" t="str">
         <v>/images/products/prod_035_1.jpg</v>
       </c>
     </row>
@@ -1425,6 +1510,9 @@
         <v>Sturdy and safe kids cycle designed for young riders (8-12 Years). Equipped with anti-skid tires, full chain guard, and ergonomic safety grips.</v>
       </c>
       <c r="K29" t="str">
+        <v>Wheel Size: 20 Inches | Frame Material: High-Tensile Carbon Steel Frame | Brake System: Calibrated Caliper Brakes with Child-Safe Levers | Gears / Speed: Single Speed Direct Drive | Front Suspension: Rigid Aerodynamic Steel Fork | Target Age Group: 8-12 Years | Ideal Location: Urban Roads, Fitness Trails &amp; City Commuting</v>
+      </c>
+      <c r="L29" t="str">
         <v>/images/products/prod_036_1.jpg</v>
       </c>
     </row>
@@ -1460,6 +1548,9 @@
         <v>Sturdy and safe kids cycle designed for young riders (5-8 Years). Equipped with anti-skid tires, full chain guard, and ergonomic safety grips.</v>
       </c>
       <c r="K30" t="str">
+        <v>Wheel Size: 16 Inches | Frame Material: High-Tensile Carbon Steel Frame | Brake System: Calibrated Caliper Brakes with Child-Safe Levers | Gears / Speed: Single Speed Direct Drive | Front Suspension: Rigid Aerodynamic Steel Fork | Target Age Group: 5-8 Years | Ideal Location: Urban Roads, Fitness Trails &amp; City Commuting</v>
+      </c>
+      <c r="L30" t="str">
         <v>/images/products/prod_037_1.jpg</v>
       </c>
     </row>
@@ -1495,6 +1586,9 @@
         <v>Durable and stylish adult cycle engineered with High-Tensile Carbon Steel Frame, Dual Mechanical Disc Brakes (Front &amp; Rear), and sleek geometry for daily commutes and fitness rides.</v>
       </c>
       <c r="K31" t="str">
+        <v>Wheel Size: 24 Inches | Frame Material: High-Tensile Carbon Steel Frame | Brake System: Dual Mechanical Disc Brakes (Front &amp; Rear) | Gears / Speed: Single Speed Direct Drive | Front Suspension: Front Telescopic Suspension Fork | Target Age Group: 12-15 Years | Ideal Location: Urban Roads, Fitness Trails &amp; City Commuting</v>
+      </c>
+      <c r="L31" t="str">
         <v>/images/products/prod_030_1_1qVziSjWYCGFf8R3oIKmAzKjvcNZu0KnG.jpg</v>
       </c>
     </row>
@@ -1530,6 +1624,9 @@
         <v>Durable and stylish adult cycle engineered with High-Tensile Carbon Steel Frame, Dual Mechanical Disc Brakes (Front &amp; Rear), and sleek geometry for daily commutes and fitness rides.</v>
       </c>
       <c r="K32" t="str">
+        <v>Wheel Size: 26 Inches | Frame Material: High-Tensile Carbon Steel Frame | Brake System: Dual Mechanical Disc Brakes (Front &amp; Rear) | Gears / Speed: Single Speed Direct Drive | Front Suspension: Front Telescopic Suspension Fork | Target Age Group: 15+ Years | Ideal Location: Urban Roads, Fitness Trails &amp; City Commuting</v>
+      </c>
+      <c r="L32" t="str">
         <v>/images/products/prod_040_1_1g-pYq_s7n50qf5m2eJN9l5r_v4edU99Z.jpg</v>
       </c>
     </row>
@@ -1565,6 +1662,9 @@
         <v>Durable and stylish adult cycle engineered with High-Tensile Carbon Steel Frame, High-Performance V-Brake System, and sleek geometry for daily commutes and fitness rides.</v>
       </c>
       <c r="K33" t="str">
+        <v>Wheel Size: 24 Inches | Frame Material: High-Tensile Carbon Steel Frame | Brake System: High-Performance V-Brake System | Gears / Speed: Single Speed Direct Drive | Front Suspension: Rigid Aerodynamic Steel Fork | Target Age Group: 12-15 Years | Ideal Location: Urban Roads, Fitness Trails &amp; City Commuting</v>
+      </c>
+      <c r="L33" t="str">
         <v>/images/products/prod_032_1_1rYYvmQpehc6qpBH7YOz0jT_aI1uTEsOQ.jpg,/images/products/prod_032_2_1qSfD9okHkQmY7E8OFcqcUlRURRiPHH8D.jpg</v>
       </c>
     </row>
@@ -1600,6 +1700,9 @@
         <v>High-performance geared cycle built with 21-Speed Gear System (Shimano / Microshift), Dual Mechanical Disc Brakes (Front &amp; Rear), and a rigid High-Tensile Carbon Steel Frame for fast city and trail riding.</v>
       </c>
       <c r="K34" t="str">
+        <v>Wheel Size: 26 Inches | Frame Material: High-Tensile Carbon Steel Frame | Brake System: Dual Mechanical Disc Brakes (Front &amp; Rear) | Gears / Speed: 21-Speed Gear System (Shimano / Microshift) | Front Suspension: Front Telescopic Suspension Fork | Target Age Group: 15+ Years | Ideal Location: Urban Roads, Fitness Trails &amp; City Commuting</v>
+      </c>
+      <c r="L34" t="str">
         <v>/images/products/prod_042_1_1VGfMRvQitXL1aQYdeM933R_pw4jiJXss.jpg</v>
       </c>
     </row>
@@ -1635,6 +1738,9 @@
         <v>Hercules Shurveer EC is an advanced electric bicycle powered by a high-torque BLDC hub motor and removable lithium battery, designed for long-range commutes across Tirunelveli.</v>
       </c>
       <c r="K35" t="str">
+        <v>Wheel Size: Standard Size | Frame Material: High-Tensile Carbon Steel Frame | Brake System: Front &amp; Rear Mechanical Power Brakes | Gears / Speed: Single Speed Direct Drive | Front Suspension: Rigid Aerodynamic Steel Fork | Target Age Group: 15+ Years | Ideal Location: Urban Roads, Fitness Trails &amp; City Commuting | Motor Type: 36V 250W High-Torque Rear Hub BLDC Motor | Battery Unit: Removable 36V Lithium-Ion LFP Battery Pack | Riding Modes: Pedal Assist (PAS) &amp; Pure Throttle Mode | Top Speed: Up to 25 km/h</v>
+      </c>
+      <c r="L35" t="str">
         <v>/images/products/prod_043_1_18abkEN_bcgrKPFHkF5ttxu6aWRIccoNj.jpg</v>
       </c>
     </row>
@@ -1670,6 +1776,9 @@
         <v>Raleigh E-surge S/s Eco is an advanced electric bicycle powered by a high-torque BLDC hub motor and removable lithium battery, designed for long-range commutes across Tirunelveli.</v>
       </c>
       <c r="K36" t="str">
+        <v>Wheel Size: Standard Size | Frame Material: Lightweight Aircraft-Grade Alloy Frame | Brake System: Front &amp; Rear Mechanical Power Brakes | Gears / Speed: Single Speed Direct Drive | Front Suspension: Rigid Aerodynamic Steel Fork | Target Age Group: 15+ Years | Ideal Location: Urban Roads, Fitness Trails &amp; City Commuting | Motor Type: 36V 250W High-Torque Rear Hub BLDC Motor | Battery Unit: Removable 36V Lithium-Ion LFP Battery Pack | Riding Modes: Pedal Assist (PAS) &amp; Pure Throttle Mode | Top Speed: Up to 25 km/h</v>
+      </c>
+      <c r="L36" t="str">
         <v>/images/products/prod_044_1.jpg</v>
       </c>
     </row>
@@ -1705,6 +1814,9 @@
         <v>Sturdy and safe kids cycle designed for young riders (8-12 Years). Equipped with anti-skid tires, full chain guard, and ergonomic safety grips.</v>
       </c>
       <c r="K37" t="str">
+        <v>Wheel Size: 20 Inches | Frame Material: High-Tensile Carbon Steel Frame | Brake System: Calibrated Caliper Brakes with Child-Safe Levers | Gears / Speed: Single Speed Direct Drive | Front Suspension: Rigid Aerodynamic Steel Fork | Target Age Group: 8-12 Years | Ideal Location: Urban Roads, Fitness Trails &amp; City Commuting</v>
+      </c>
+      <c r="L37" t="str">
         <v>/images/products/prod_046_1_12-l0LZzxDB78A0b3ENPw61IPM1TbNp-e.jpg</v>
       </c>
     </row>
@@ -1740,6 +1852,9 @@
         <v>Elegant and comfortable girls cycle featuring low step-through frame, comfortable upright geometry, rear carrier, and smooth brake controls.</v>
       </c>
       <c r="K38" t="str">
+        <v>Wheel Size: 24 Inches | Frame Material: High-Tensile Carbon Steel Frame | Brake System: Front &amp; Rear Mechanical Power Brakes | Gears / Speed: Single Speed Direct Drive | Front Suspension: Rigid Aerodynamic Steel Fork | Target Age Group: 12-15 Years | Ideal Location: Urban Roads, Fitness Trails &amp; City Commuting</v>
+      </c>
+      <c r="L38" t="str">
         <v>/images/products/prod_047_1_12dXbchyMT1JX3me2LR2NMcyZY9LlvDvG.jpg,/images/products/prod_047_2_1ZloQm8BkEBmS1dycx5Gt0-2Pkmm4oW7k.jpg</v>
       </c>
     </row>
@@ -1775,6 +1890,9 @@
         <v>Durable and stylish adult cycle engineered with Lightweight Aircraft-Grade Alloy Frame, Dual Mechanical Disc Brakes (Front &amp; Rear), and sleek geometry for daily commutes and fitness rides.</v>
       </c>
       <c r="K39" t="str">
+        <v>Wheel Size: 26 Inches | Frame Material: Lightweight Aircraft-Grade Alloy Frame | Brake System: Dual Mechanical Disc Brakes (Front &amp; Rear) | Gears / Speed: Single Speed Direct Drive | Front Suspension: Front Telescopic Suspension Fork | Target Age Group: 15+ Years | Ideal Location: Urban Roads, Fitness Trails &amp; City Commuting</v>
+      </c>
+      <c r="L39" t="str">
         <v>/images/products/prod_048_1_1q9hYp6kdJYhpvmBvWxFKHGGbUYovFiXh.jpg</v>
       </c>
     </row>
@@ -1810,6 +1928,9 @@
         <v>Durable and stylish adult cycle engineered with Lightweight Aircraft-Grade Alloy Frame, Front &amp; Rear Mechanical Power Brakes, and sleek geometry for daily commutes and fitness rides.</v>
       </c>
       <c r="K40" t="str">
+        <v>Wheel Size: 29 Inches | Frame Material: Lightweight Aircraft-Grade Alloy Frame | Brake System: Front &amp; Rear Mechanical Power Brakes | Gears / Speed: Single Speed Direct Drive | Front Suspension: Rigid Aerodynamic Steel Fork | Target Age Group: 15+ Years | Ideal Location: Urban Roads, Fitness Trails &amp; City Commuting</v>
+      </c>
+      <c r="L40" t="str">
         <v>/images/products/prod_049_1_17DZ0XXndgxQv-Za--OftlEZ4Jo9MLJLK.jpg,/images/products/prod_049_2_1qV2Wmetczbft1-kyA6E2yKZ-X_QJYHWM.jpg</v>
       </c>
     </row>
@@ -1845,6 +1966,9 @@
         <v>High-performance geared cycle built with 21-Speed Gear System (Shimano / Microshift), Front &amp; Rear Mechanical Power Brakes, and a rigid Lightweight Aircraft-Grade Alloy Frame for fast city and trail riding.</v>
       </c>
       <c r="K41" t="str">
+        <v>Wheel Size: 29 Inches | Frame Material: Lightweight Aircraft-Grade Alloy Frame | Brake System: Front &amp; Rear Mechanical Power Brakes | Gears / Speed: 21-Speed Gear System (Shimano / Microshift) | Front Suspension: Rigid Aerodynamic Steel Fork | Target Age Group: 15+ Years | Ideal Location: Urban Roads, Fitness Trails &amp; City Commuting</v>
+      </c>
+      <c r="L41" t="str">
         <v>/images/products/prod_052_1_105NvCgjVtXGtaeqUeDr858YjfsaNBmNa.jpg</v>
       </c>
     </row>
@@ -1880,6 +2004,9 @@
         <v>High-performance geared cycle built with Multi-Speed Gear System, Dual Mechanical Disc Brakes (Front &amp; Rear), and a rigid High-Tensile Carbon Steel Frame for fast city and trail riding.</v>
       </c>
       <c r="K42" t="str">
+        <v>Wheel Size: Standard Size | Frame Material: High-Tensile Carbon Steel Frame | Brake System: Dual Mechanical Disc Brakes (Front &amp; Rear) | Gears / Speed: Multi-Speed Gear System | Front Suspension: Front Telescopic Suspension Fork | Target Age Group: 15+ Years | Ideal Location: Urban Roads, Fitness Trails &amp; City Commuting</v>
+      </c>
+      <c r="L42" t="str">
         <v>/images/products/prod_054_1.jpg</v>
       </c>
     </row>
@@ -1915,6 +2042,9 @@
         <v>AOKI Street Mamba is an advanced electric bicycle powered by a high-torque BLDC hub motor and removable lithium battery, designed for long-range commutes across Tirunelveli.</v>
       </c>
       <c r="K43" t="str">
+        <v>Wheel Size: Standard Size | Frame Material: High-Tensile Carbon Steel Frame | Brake System: Front &amp; Rear Mechanical Power Brakes | Gears / Speed: Single Speed Direct Drive | Front Suspension: Rigid Aerodynamic Steel Fork | Target Age Group: 15+ Years | Ideal Location: Urban Roads, Fitness Trails &amp; City Commuting | Motor Type: 36V 250W High-Torque Rear Hub BLDC Motor | Battery Unit: Removable 36V Lithium-Ion LFP Battery Pack | Riding Modes: Pedal Assist (PAS) &amp; Pure Throttle Mode | Top Speed: Up to 25 km/h</v>
+      </c>
+      <c r="L43" t="str">
         <v>/images/products/prod_055_1.jpg,/images/products/prod_055_2.jpg</v>
       </c>
     </row>
@@ -1950,6 +2080,9 @@
         <v>Durable and stylish adult cycle engineered with Lightweight Aircraft-Grade Alloy Frame, Front &amp; Rear Mechanical Power Brakes, and sleek geometry for daily commutes and fitness rides.</v>
       </c>
       <c r="K44" t="str">
+        <v>Wheel Size: 29 Inches | Frame Material: Lightweight Aircraft-Grade Alloy Frame | Brake System: Front &amp; Rear Mechanical Power Brakes | Gears / Speed: Single Speed Direct Drive | Front Suspension: Rigid Aerodynamic Steel Fork | Target Age Group: 15+ Years | Ideal Location: Urban Roads, Fitness Trails &amp; City Commuting</v>
+      </c>
+      <c r="L44" t="str">
         <v>/images/products/prod_056_1_1Ws3eOH-sOZouOZB14wePKR-eqO69kGwH.jpg</v>
       </c>
     </row>
@@ -1985,6 +2118,9 @@
         <v>Durable and stylish adult cycle engineered with High-Tensile Carbon Steel Frame, Dual Mechanical Disc Brakes (Front &amp; Rear), and sleek geometry for daily commutes and fitness rides.</v>
       </c>
       <c r="K45" t="str">
+        <v>Wheel Size: 26 Inches | Frame Material: High-Tensile Carbon Steel Frame | Brake System: Dual Mechanical Disc Brakes (Front &amp; Rear) | Gears / Speed: Single Speed Direct Drive | Front Suspension: Front Telescopic Suspension Fork | Target Age Group: 15+ Years | Ideal Location: Urban Roads, Fitness Trails &amp; City Commuting</v>
+      </c>
+      <c r="L45" t="str">
         <v>/images/products/prod_057_1_1k1yFIJJdHeoq9OAfD4q2lDOsT0I7j1Mf.jpg,/images/products/prod_057_2_1iPIByYnUQzn3NtdOw85C-0Tfd93VRUsN.jpg</v>
       </c>
     </row>
@@ -2020,6 +2156,9 @@
         <v>Durable and stylish adult cycle engineered with High-Tensile Carbon Steel Frame, High-Performance V-Brake System, and sleek geometry for daily commutes and fitness rides.</v>
       </c>
       <c r="K46" t="str">
+        <v>Wheel Size: 24 Inches | Frame Material: High-Tensile Carbon Steel Frame | Brake System: High-Performance V-Brake System | Gears / Speed: Single Speed Direct Drive | Front Suspension: Rigid Aerodynamic Steel Fork | Target Age Group: 12-15 Years | Ideal Location: Urban Roads, Fitness Trails &amp; City Commuting</v>
+      </c>
+      <c r="L46" t="str">
         <v>/images/products/prod_058_1_19hv2ju_nqrZGcVFJCD0fotD41RiwWNuc.jpg,/images/products/prod_058_2_1OT8rO3PDeCLBzsLHMUWJ_UyCckcc6lX2.jpg</v>
       </c>
     </row>
@@ -2055,6 +2194,9 @@
         <v>Durable and stylish adult cycle engineered with High-Tensile Carbon Steel Frame, Dual Mechanical Disc Brakes (Front &amp; Rear), and sleek geometry for daily commutes and fitness rides.</v>
       </c>
       <c r="K47" t="str">
+        <v>Wheel Size: 24 Inches | Frame Material: High-Tensile Carbon Steel Frame | Brake System: Dual Mechanical Disc Brakes (Front &amp; Rear) | Gears / Speed: Single Speed Direct Drive | Front Suspension: Front Telescopic Suspension Fork | Target Age Group: 12-15 Years | Ideal Location: Urban Roads, Fitness Trails &amp; City Commuting</v>
+      </c>
+      <c r="L47" t="str">
         <v>https://drive.google.com/file/d//view?usp=sharing,/images/products/prod_057_2_1iPIByYnUQzn3NtdOw85C-0Tfd93VRUsN.jpg,/images/products/prod_057_2_1iPIByYnUQzn3NtdOw85C-0Tfd93VRUsN.jpg</v>
       </c>
     </row>
@@ -2090,6 +2232,9 @@
         <v>Durable and stylish adult cycle engineered with Lightweight Aircraft-Grade Alloy Frame, Front &amp; Rear Mechanical Power Brakes, and sleek geometry for daily commutes and fitness rides.</v>
       </c>
       <c r="K48" t="str">
+        <v>Wheel Size: 29 Inches | Frame Material: Lightweight Aircraft-Grade Alloy Frame | Brake System: Front &amp; Rear Mechanical Power Brakes | Gears / Speed: Single Speed Direct Drive | Front Suspension: Rigid Aerodynamic Steel Fork | Target Age Group: 15+ Years | Ideal Location: Urban Roads, Fitness Trails &amp; City Commuting</v>
+      </c>
+      <c r="L48" t="str">
         <v>/images/products/prod_062_1.jpg</v>
       </c>
     </row>
@@ -2125,6 +2270,9 @@
         <v>AOKI Street Gost is an advanced electric bicycle powered by a high-torque BLDC hub motor and removable lithium battery, designed for long-range commutes across Tirunelveli.</v>
       </c>
       <c r="K49" t="str">
+        <v>Wheel Size: Standard Size | Frame Material: High-Tensile Carbon Steel Frame | Brake System: Front &amp; Rear Mechanical Power Brakes | Gears / Speed: Single Speed Direct Drive | Front Suspension: Rigid Aerodynamic Steel Fork | Target Age Group: 15+ Years | Ideal Location: Urban Roads, Fitness Trails &amp; City Commuting | Motor Type: 36V 250W High-Torque Rear Hub BLDC Motor | Battery Unit: Removable 36V Lithium-Ion LFP Battery Pack | Riding Modes: Pedal Assist (PAS) &amp; Pure Throttle Mode | Top Speed: Up to 25 km/h</v>
+      </c>
+      <c r="L49" t="str">
         <v>/images/products/prod_064_1.jpg</v>
       </c>
     </row>
@@ -2160,6 +2308,9 @@
         <v>Hercules Hardstyle 27.5t EC Non Sus DD is an advanced electric bicycle powered by a high-torque BLDC hub motor and removable lithium battery, designed for long-range commutes across Tirunelveli.</v>
       </c>
       <c r="K50" t="str">
+        <v>Wheel Size: 27.5 Inches | Frame Material: High-Tensile Carbon Steel Frame | Brake System: Dual Mechanical Disc Brakes (Front &amp; Rear) | Gears / Speed: Single Speed Direct Drive | Front Suspension: Rigid Aerodynamic Steel Fork | Target Age Group: 15+ Years | Ideal Location: Urban Roads, Fitness Trails &amp; City Commuting | Motor Type: 36V 250W High-Torque Rear Hub BLDC Motor | Battery Unit: Removable 36V Lithium-Ion LFP Battery Pack | Riding Modes: Pedal Assist (PAS) &amp; Pure Throttle Mode | Top Speed: Up to 25 km/h</v>
+      </c>
+      <c r="L50" t="str">
         <v>/images/products/prod_049_1_1ixyGkpCmUa9Md78oqjMOHj42I4tFqD0S.jpg</v>
       </c>
     </row>
@@ -2195,6 +2346,9 @@
         <v>Durable and stylish adult cycle engineered with Lightweight Aircraft-Grade Alloy Frame, Dual Mechanical Disc Brakes (Front &amp; Rear), and sleek geometry for daily commutes and fitness rides.</v>
       </c>
       <c r="K51" t="str">
+        <v>Wheel Size: 29 Inches | Frame Material: Lightweight Aircraft-Grade Alloy Frame | Brake System: Dual Mechanical Disc Brakes (Front &amp; Rear) | Gears / Speed: Single Speed Direct Drive | Front Suspension: Front Telescopic Suspension Fork | Target Age Group: 15+ Years | Ideal Location: Urban Roads, Fitness Trails &amp; City Commuting</v>
+      </c>
+      <c r="L51" t="str">
         <v>/images/products/prod_050_1_168Y_oxmz0eUB7UldAykn2oXjREuOzDWJ.jpg,/images/products/prod_050_2_13OKzmHpJoh0_SJpkc89YiaGslaRe_ivZ.jpg</v>
       </c>
     </row>
@@ -2230,12 +2384,15 @@
         <v>Beeride Luminious 26T FSDD is an advanced electric bicycle powered by a high-torque BLDC hub motor and removable lithium battery, designed for long-range commutes across Tirunelveli.</v>
       </c>
       <c r="K52" t="str">
+        <v>Wheel Size: 26 Inches | Frame Material: High-Tensile Carbon Steel Frame | Brake System: Dual Mechanical Disc Brakes (Front &amp; Rear) | Gears / Speed: Single Speed Direct Drive | Front Suspension: Front Telescopic Suspension Fork | Target Age Group: 15+ Years | Ideal Location: Urban Roads, Fitness Trails &amp; City Commuting | Motor Type: 36V 250W High-Torque Rear Hub BLDC Motor | Battery Unit: Removable 36V Lithium-Ion LFP Battery Pack | Riding Modes: Pedal Assist (PAS) &amp; Pure Throttle Mode | Top Speed: Up to 25 km/h</v>
+      </c>
+      <c r="L52" t="str">
         <v>/images/products/prod_051_1_1DofcHHbhKLTZgifImBQg5JxfboSO0BGC.jpg</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:K52"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:L52"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Branch: NEXT-PRE-DEVELOPMENT - feat: update product images and inventory data
</commit_message>
<xml_diff>
--- a/store_inventory_template.xlsx
+++ b/store_inventory_template.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="738" uniqueCount="338">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="759" uniqueCount="347">
   <si>
     <t>product_id</t>
   </si>
@@ -1214,7 +1214,7 @@
     <t>Wheel Size: 26 Inches | Frame Material: High-Tensile  Steel Frame | Brake System: Front &amp; Rear Mechanical Power Brakes | Gears / Speed: Multi-Speed Gear System | Front Suspension: Suspension Steel Fork | Target Age Group: 15+ Years | Ideal Location: Urban Roads, Fitness Trails &amp; City Commuting | Tire Dimensions: 26 x 4.0 Inch Ultra-Wide All-Terrain Tread</t>
   </si>
   <si>
-    <t>/images/products/prod_052_1_105NvCgjVtXGtaeqUeDr858YjfsaNBmNa.jpg</t>
+    <t>/images/products/prod_052_1_105NvCgjVtXGtaeqUeDr858YjfsaNBmNa.jpg,images/products/prod_024_2.jpg,</t>
   </si>
   <si>
     <t>prod_059</t>
@@ -1349,19 +1349,31 @@
     <t>prod_065</t>
   </si>
   <si>
-    <t>RALEIGH NAVARRO ONE 29T SS</t>
+    <t>SUNCROSS TOSCANO (21 SPEED) ALLOY</t>
+  </si>
+  <si>
+    <t>Wheel Size: 29 Inches | Frame Material: High-Tensile Alloy  Steel Frame | Brake System: Dual Mechanical Disc Brakes (Front &amp; Rear) | Gears / Speed: 21Speed Direct Drive | Front Suspension: Front Telescopic Suspension Fork | Target Age Group: 15+ Years | Ideal Location: Urban Roads, Fitness Trails &amp; City Commuting</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/file/d/1h6UEG4cGPgSi-oYXiNYmzuQLxD_Y5p-Q/view?usp=sharing</t>
+  </si>
+  <si>
+    <t>prod_066</t>
+  </si>
+  <si>
+    <t>RALEIGH AVALANCHE 27.5T</t>
   </si>
   <si>
     <t>Durable and stylish adult cycle engineered with Hi-Ten Steel with Internal Cable Routing Frame, Dual Mechanical Disc Brakes (Front &amp; Rear), and sleek geometry for daily commutes and fitness rides.</t>
   </si>
   <si>
-    <t>Wheel Size: 29 Inches | Frame Material: High-Tensile  Steel Frame Frame | Brake System: Dual Mechanical Disc Brakes| Gears / Speed: Single Speed Direct Drive | Front Suspension: Suspension  Fork | Target Age Group: 15+ Years | Ideal Location: Urban Roads, Fitness Trails &amp; City Commuting</t>
-  </si>
-  <si>
-    <t>/images/products/prod_056_1_1Ws3eOH-sOZouOZB14wePKR-eqO69kGwH.jpg</t>
-  </si>
-  <si>
-    <t>prod_066</t>
+    <t>Wheel Size: 27.5T Inches | Frame Material: High-Tensile  Steel Frame Frame | Brake System: Dual Mechanical Disc Brakes| Gears / Speed: Single Speed Direct Drive | Front Suspension: Suspension  Fork | Target Age Group: 15+ Years | Ideal Location: Urban Roads, Fitness Trails &amp; City Commuting</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/file/d/1vwrVwG-FmGwAcVKAPCRwA8A1OGRX6OvW/view?usp=sharing</t>
+  </si>
+  <si>
+    <t>prod_067</t>
   </si>
   <si>
     <t>RALEIGH PHASE PRO 29T S/S</t>
@@ -1373,7 +1385,7 @@
     <t>/images/products/prod_062_1.jpg</t>
   </si>
   <si>
-    <t>prod_067</t>
+    <t>prod_068</t>
   </si>
   <si>
     <t>RALEIGH EXALT 29T SS</t>
@@ -1385,7 +1397,7 @@
     <t>/images/products/prod_049_1_17DZ0XXndgxQv-Za--OftlEZ4Jo9MLJLK.jpg,/images/products/prod_049_2_1qV2Wmetczbft1-kyA6E2yKZ-X_QJYHWM.jpg</t>
   </si>
   <si>
-    <t>prod_068</t>
+    <t>prod_069</t>
   </si>
   <si>
     <t>RALEIGH NAVARRO ONE 29T (D/Disc)</t>
@@ -1394,10 +1406,10 @@
     <t>Wheel Size: 29 Inches | Frame Material:High-Tensile  Steel Frame | | Brake System: Dual Mechanical Disc Brakes (Front &amp; Rear) | Gears / Speed: Single Speed Direct Drive | Front Suspension: Suspension Fork | Target Age Group: 15+ Years | Ideal Location: Urban Roads, Fitness Trails &amp; City Commuting</t>
   </si>
   <si>
-    <t>/images/products/prod_024_1.jpg,/images/products/prod_024_2.jpg,/images/products/prod_024_3.jpg</t>
-  </si>
-  <si>
-    <t>prod_069</t>
+    <t>/images/products/prod_024_1.jpg,/images/products/prod_024_3.jpg</t>
+  </si>
+  <si>
+    <t>prod_070</t>
   </si>
   <si>
     <t>RALEIGH CAPTUS 29T FSDD SS</t>
@@ -1409,7 +1421,7 @@
     <t>/images/products/prod_050_1_168Y_oxmz0eUB7UldAykn2oXjREuOzDWJ.jpg,/images/products/prod_050_2_13OKzmHpJoh0_SJpkc89YiaGslaRe_ivZ.jpg</t>
   </si>
   <si>
-    <t>prod_070</t>
+    <t>prod_071</t>
   </si>
   <si>
     <t>LUCIFIRE P Pro 12 29T</t>
@@ -1419,6 +1431,70 @@
   </si>
   <si>
     <t>Durable and stylish adult cycle engineered with Lightweight Aircraft-Grade Alloy Frame, Front &amp; Rear Mechanical Disc Brakes, and sleek geometry for daily commutes and fitness rides.</t>
+  </si>
+  <si>
+    <t>Wheel Size: 29 Inches | Frame Material: High-Tensile Alloy  Steel Frame | Brake System: Dual Mechanical Disc Brakes (Front &amp; Rear) | Gears / Speed: Single Speed Direct Drive | Front Suspension: Front Telescopic Suspension Fork | Target Age Group: 15+ Years | Ideal Location: Urban Roads, Fitness Trails &amp; City Commuting</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <color rgb="FF1155CC"/>
+        <u/>
+      </rPr>
+      <t>https://drive.google.com/file/d/127LKOEq44jMf3WgQ2mXYjDrPtVDvqcEm/view?usp=sharing</t>
+    </r>
+    <r>
+      <rPr/>
+      <t>,</t>
+    </r>
+    <r>
+      <rPr>
+        <color rgb="FF1155CC"/>
+        <u/>
+      </rPr>
+      <t>https://drive.google.com/file/d/1dYpBo_0kJConVPzMcXPBkYNr-maCmwAh/view?usp=sharing</t>
+    </r>
+  </si>
+  <si>
+    <t>prod_072</t>
+  </si>
+  <si>
+    <t>LUCIFIRE Morpheus 29T</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <color rgb="FF1155CC"/>
+        <u/>
+      </rPr>
+      <t>https://drive.google.com/file/d/1sTpQlE2fZZjItcmXNZQLDc1GeMYBO8qF/view?usp=sharing</t>
+    </r>
+    <r>
+      <rPr/>
+      <t>,</t>
+    </r>
+    <r>
+      <rPr>
+        <color rgb="FF1155CC"/>
+        <u/>
+      </rPr>
+      <t>https://drive.google.com/file/d/10orTYGKpp5M1GbLDJroOK3zVOm9DC5EZ/view?usp=sharing</t>
+    </r>
+    <r>
+      <rPr/>
+      <t>,</t>
+    </r>
+    <r>
+      <rPr>
+        <color rgb="FF1155CC"/>
+        <u/>
+      </rPr>
+      <t>https://drive.google.com/file/d/1bJmsmm8f3_GlmsgFBroHEsYtnGzF_Ewd/view?usp=sharing</t>
+    </r>
+    <r>
+      <rPr/>
+      <t>,https://drive.google.com/file/d/1bJmsmm8f3_GlmsgFBroHEsYtnGzF_Ewd/view?usp=sharing</t>
+    </r>
   </si>
   <si>
     <t>slug</t>
@@ -1485,7 +1561,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <fonts count="7">
+  <fonts count="8">
     <font>
       <sz val="12.0"/>
       <color theme="1"/>
@@ -1520,6 +1596,12 @@
       <color rgb="FF0000FF"/>
       <name val="Calibri"/>
     </font>
+    <font>
+      <u/>
+      <sz val="12.0"/>
+      <color rgb="FF0000FF"/>
+      <name val="Calibri"/>
+    </font>
   </fonts>
   <fills count="3">
     <fill>
@@ -1541,7 +1623,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="12">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -1571,6 +1653,9 @@
       <alignment horizontal="right" readingOrder="0" vertical="bottom"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0" vertical="bottom"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" vertical="bottom"/>
     </xf>
   </cellXfs>
@@ -4084,7 +4169,7 @@
       <c r="K59" s="8" t="s">
         <v>262</v>
       </c>
-      <c r="L59" s="1" t="s">
+      <c r="L59" s="2" t="s">
         <v>263</v>
       </c>
     </row>
@@ -4362,38 +4447,38 @@
       <c r="A66" s="1" t="s">
         <v>293</v>
       </c>
-      <c r="B66" s="6" t="s">
+      <c r="B66" s="2" t="s">
         <v>294</v>
       </c>
-      <c r="C66" s="6" t="s">
-        <v>212</v>
-      </c>
-      <c r="D66" s="6" t="s">
-        <v>34</v>
-      </c>
-      <c r="E66" s="6" t="s">
+      <c r="C66" s="8" t="s">
+        <v>276</v>
+      </c>
+      <c r="D66" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="E66" s="8" t="s">
         <v>260</v>
       </c>
-      <c r="F66" s="7">
-        <v>13000.0</v>
-      </c>
-      <c r="G66" s="7">
-        <v>12500.0</v>
+      <c r="F66" s="9">
+        <v>23000.0</v>
+      </c>
+      <c r="G66" s="9">
+        <v>21000.0</v>
       </c>
       <c r="H66" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="I66" s="6" t="s">
+      <c r="I66" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="J66" s="8" t="s">
+      <c r="J66" s="2" t="s">
+        <v>282</v>
+      </c>
+      <c r="K66" s="8" t="s">
         <v>295</v>
       </c>
-      <c r="K66" s="8" t="s">
+      <c r="L66" s="11" t="s">
         <v>296</v>
-      </c>
-      <c r="L66" s="6" t="s">
-        <v>297</v>
       </c>
       <c r="M66" s="6"/>
       <c r="N66" s="6"/>
@@ -4412,10 +4497,10 @@
     </row>
     <row r="67">
       <c r="A67" s="2" t="s">
+        <v>297</v>
+      </c>
+      <c r="B67" s="8" t="s">
         <v>298</v>
-      </c>
-      <c r="B67" s="6" t="s">
-        <v>299</v>
       </c>
       <c r="C67" s="6" t="s">
         <v>212</v>
@@ -4423,14 +4508,14 @@
       <c r="D67" s="6" t="s">
         <v>34</v>
       </c>
-      <c r="E67" s="6" t="s">
-        <v>260</v>
-      </c>
-      <c r="F67" s="7">
-        <v>13100.0</v>
-      </c>
-      <c r="G67" s="7">
-        <v>12800.0</v>
+      <c r="E67" s="1" t="s">
+        <v>213</v>
+      </c>
+      <c r="F67" s="9">
+        <v>15000.0</v>
+      </c>
+      <c r="G67" s="9">
+        <v>13900.0</v>
       </c>
       <c r="H67" s="6" t="s">
         <v>17</v>
@@ -4439,12 +4524,12 @@
         <v>18</v>
       </c>
       <c r="J67" s="8" t="s">
-        <v>295</v>
+        <v>299</v>
       </c>
       <c r="K67" s="8" t="s">
         <v>300</v>
       </c>
-      <c r="L67" s="6" t="s">
+      <c r="L67" s="11" t="s">
         <v>301</v>
       </c>
       <c r="M67" s="6"/>
@@ -4462,45 +4547,59 @@
       <c r="Y67" s="6"/>
       <c r="Z67" s="6"/>
     </row>
-    <row r="68" ht="15.75" customHeight="1">
+    <row r="68">
       <c r="A68" s="1" t="s">
         <v>302</v>
       </c>
-      <c r="B68" s="1" t="s">
+      <c r="B68" s="6" t="s">
         <v>303</v>
       </c>
-      <c r="C68" s="1" t="s">
+      <c r="C68" s="6" t="s">
         <v>212</v>
       </c>
-      <c r="D68" s="1" t="s">
+      <c r="D68" s="6" t="s">
         <v>34</v>
       </c>
-      <c r="E68" s="1" t="s">
+      <c r="E68" s="6" t="s">
         <v>260</v>
       </c>
-      <c r="F68" s="1">
-        <v>13995.0</v>
-      </c>
-      <c r="G68" s="1">
-        <v>13500.0</v>
-      </c>
-      <c r="H68" s="1" t="s">
+      <c r="F68" s="7">
+        <v>13100.0</v>
+      </c>
+      <c r="G68" s="7">
+        <v>12800.0</v>
+      </c>
+      <c r="H68" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="I68" s="1" t="s">
+      <c r="I68" s="6" t="s">
         <v>18</v>
       </c>
       <c r="J68" s="8" t="s">
-        <v>295</v>
-      </c>
-      <c r="K68" s="2" t="s">
+        <v>299</v>
+      </c>
+      <c r="K68" s="8" t="s">
         <v>304</v>
       </c>
-      <c r="L68" s="1" t="s">
+      <c r="L68" s="6" t="s">
         <v>305</v>
       </c>
-    </row>
-    <row r="69">
+      <c r="M68" s="6"/>
+      <c r="N68" s="6"/>
+      <c r="O68" s="6"/>
+      <c r="P68" s="6"/>
+      <c r="Q68" s="6"/>
+      <c r="R68" s="6"/>
+      <c r="S68" s="6"/>
+      <c r="T68" s="6"/>
+      <c r="U68" s="6"/>
+      <c r="V68" s="6"/>
+      <c r="W68" s="6"/>
+      <c r="X68" s="6"/>
+      <c r="Y68" s="6"/>
+      <c r="Z68" s="6"/>
+    </row>
+    <row r="69" ht="15.75" customHeight="1">
       <c r="A69" s="2" t="s">
         <v>306</v>
       </c>
@@ -4517,19 +4616,19 @@
         <v>260</v>
       </c>
       <c r="F69" s="1">
-        <v>14175.0</v>
+        <v>13995.0</v>
       </c>
       <c r="G69" s="1">
-        <v>13925.0</v>
+        <v>13500.0</v>
       </c>
       <c r="H69" s="1" t="s">
-        <v>25</v>
+        <v>17</v>
       </c>
       <c r="I69" s="1" t="s">
         <v>18</v>
       </c>
       <c r="J69" s="8" t="s">
-        <v>295</v>
+        <v>299</v>
       </c>
       <c r="K69" s="2" t="s">
         <v>308</v>
@@ -4538,67 +4637,53 @@
         <v>309</v>
       </c>
     </row>
-    <row r="70" ht="15.75" customHeight="1">
+    <row r="70">
       <c r="A70" s="1" t="s">
         <v>310</v>
       </c>
-      <c r="B70" s="6" t="s">
+      <c r="B70" s="1" t="s">
         <v>311</v>
       </c>
-      <c r="C70" s="6" t="s">
+      <c r="C70" s="1" t="s">
         <v>212</v>
       </c>
-      <c r="D70" s="6" t="s">
+      <c r="D70" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="E70" s="6" t="s">
+      <c r="E70" s="1" t="s">
         <v>260</v>
       </c>
-      <c r="F70" s="7">
-        <v>15900.0</v>
-      </c>
-      <c r="G70" s="7">
-        <v>14900.0</v>
-      </c>
-      <c r="H70" s="6" t="s">
+      <c r="F70" s="1">
+        <v>14175.0</v>
+      </c>
+      <c r="G70" s="1">
+        <v>13925.0</v>
+      </c>
+      <c r="H70" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="I70" s="6" t="s">
+      <c r="I70" s="1" t="s">
         <v>18</v>
       </c>
       <c r="J70" s="8" t="s">
-        <v>295</v>
-      </c>
-      <c r="K70" s="8" t="s">
+        <v>299</v>
+      </c>
+      <c r="K70" s="2" t="s">
         <v>312</v>
       </c>
-      <c r="L70" s="6" t="s">
+      <c r="L70" s="2" t="s">
         <v>313</v>
       </c>
-      <c r="M70" s="6"/>
-      <c r="N70" s="6"/>
-      <c r="O70" s="6"/>
-      <c r="P70" s="6"/>
-      <c r="Q70" s="6"/>
-      <c r="R70" s="6"/>
-      <c r="S70" s="6"/>
-      <c r="T70" s="6"/>
-      <c r="U70" s="6"/>
-      <c r="V70" s="6"/>
-      <c r="W70" s="6"/>
-      <c r="X70" s="6"/>
-      <c r="Y70" s="6"/>
-      <c r="Z70" s="6"/>
-    </row>
-    <row r="71">
+    </row>
+    <row r="71" ht="15.75" customHeight="1">
       <c r="A71" s="2" t="s">
         <v>314</v>
       </c>
-      <c r="B71" s="2" t="s">
+      <c r="B71" s="6" t="s">
         <v>315</v>
       </c>
-      <c r="C71" s="2" t="s">
-        <v>316</v>
+      <c r="C71" s="6" t="s">
+        <v>212</v>
       </c>
       <c r="D71" s="6" t="s">
         <v>34</v>
@@ -4606,27 +4691,119 @@
       <c r="E71" s="6" t="s">
         <v>260</v>
       </c>
-      <c r="F71" s="2">
-        <v>17200.0</v>
-      </c>
-      <c r="G71" s="2">
-        <v>16200.0</v>
-      </c>
-      <c r="H71" s="1" t="s">
-        <v>17</v>
+      <c r="F71" s="7">
+        <v>15900.0</v>
+      </c>
+      <c r="G71" s="7">
+        <v>14900.0</v>
+      </c>
+      <c r="H71" s="6" t="s">
+        <v>25</v>
       </c>
       <c r="I71" s="6" t="s">
         <v>18</v>
       </c>
       <c r="J71" s="8" t="s">
+        <v>299</v>
+      </c>
+      <c r="K71" s="8" t="s">
+        <v>316</v>
+      </c>
+      <c r="L71" s="6" t="s">
         <v>317</v>
       </c>
-      <c r="K71" s="8" t="s">
-        <v>312</v>
-      </c>
-    </row>
-    <row r="93" ht="15.75" customHeight="1"/>
-    <row r="107" ht="15.75" customHeight="1"/>
+      <c r="M71" s="6"/>
+      <c r="N71" s="6"/>
+      <c r="O71" s="6"/>
+      <c r="P71" s="6"/>
+      <c r="Q71" s="6"/>
+      <c r="R71" s="6"/>
+      <c r="S71" s="6"/>
+      <c r="T71" s="6"/>
+      <c r="U71" s="6"/>
+      <c r="V71" s="6"/>
+      <c r="W71" s="6"/>
+      <c r="X71" s="6"/>
+      <c r="Y71" s="6"/>
+      <c r="Z71" s="6"/>
+    </row>
+    <row r="72">
+      <c r="A72" s="1" t="s">
+        <v>318</v>
+      </c>
+      <c r="B72" s="2" t="s">
+        <v>319</v>
+      </c>
+      <c r="C72" s="2" t="s">
+        <v>320</v>
+      </c>
+      <c r="D72" s="6" t="s">
+        <v>34</v>
+      </c>
+      <c r="E72" s="6" t="s">
+        <v>260</v>
+      </c>
+      <c r="F72" s="2">
+        <v>17200.0</v>
+      </c>
+      <c r="G72" s="2">
+        <v>16200.0</v>
+      </c>
+      <c r="H72" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="I72" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="J72" s="8" t="s">
+        <v>321</v>
+      </c>
+      <c r="K72" s="8" t="s">
+        <v>322</v>
+      </c>
+      <c r="L72" s="3" t="s">
+        <v>323</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="2" t="s">
+        <v>324</v>
+      </c>
+      <c r="B73" s="2" t="s">
+        <v>325</v>
+      </c>
+      <c r="C73" s="2" t="s">
+        <v>320</v>
+      </c>
+      <c r="D73" s="6" t="s">
+        <v>34</v>
+      </c>
+      <c r="E73" s="6" t="s">
+        <v>260</v>
+      </c>
+      <c r="F73" s="2">
+        <v>14800.0</v>
+      </c>
+      <c r="G73" s="2">
+        <v>13800.0</v>
+      </c>
+      <c r="H73" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="I73" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="J73" s="8" t="s">
+        <v>299</v>
+      </c>
+      <c r="K73" s="8" t="s">
+        <v>316</v>
+      </c>
+      <c r="L73" s="3" t="s">
+        <v>326</v>
+      </c>
+    </row>
+    <row r="94" ht="15.75" customHeight="1"/>
     <row r="108" ht="15.75" customHeight="1"/>
     <row r="109" ht="15.75" customHeight="1"/>
     <row r="110" ht="15.75" customHeight="1"/>
@@ -5546,6 +5723,7 @@
     <row r="1024" ht="15.75" customHeight="1"/>
     <row r="1025" ht="15.75" customHeight="1"/>
     <row r="1026" ht="15.75" customHeight="1"/>
+    <row r="1027" ht="15.75" customHeight="1"/>
   </sheetData>
   <hyperlinks>
     <hyperlink r:id="rId1" ref="L3"/>
@@ -5566,8 +5744,12 @@
     <hyperlink r:id="rId16" ref="L39"/>
     <hyperlink r:id="rId17" ref="L55"/>
     <hyperlink r:id="rId18" ref="L61"/>
+    <hyperlink r:id="rId19" ref="L66"/>
+    <hyperlink r:id="rId20" ref="L67"/>
+    <hyperlink r:id="rId21" ref="L72"/>
+    <hyperlink r:id="rId22" ref="L73"/>
   </hyperlinks>
-  <drawing r:id="rId19"/>
+  <drawing r:id="rId23"/>
 </worksheet>
 </file>
 
@@ -5588,7 +5770,7 @@
         <v>1</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>318</v>
+        <v>327</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>9</v>
@@ -5599,13 +5781,13 @@
         <v>102</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>319</v>
+        <v>328</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>320</v>
+        <v>329</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>321</v>
+        <v>330</v>
       </c>
     </row>
     <row r="3">
@@ -5613,13 +5795,13 @@
         <v>34</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>322</v>
+        <v>331</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>323</v>
+        <v>332</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>324</v>
+        <v>333</v>
       </c>
     </row>
     <row r="4">
@@ -5627,13 +5809,13 @@
         <v>58</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>325</v>
+        <v>334</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>326</v>
+        <v>335</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>327</v>
+        <v>336</v>
       </c>
     </row>
     <row r="5">
@@ -5641,13 +5823,13 @@
         <v>15</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>328</v>
+        <v>337</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>329</v>
+        <v>338</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>330</v>
+        <v>339</v>
       </c>
     </row>
     <row r="6">
@@ -5655,27 +5837,27 @@
         <v>196</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>331</v>
+        <v>340</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>332</v>
+        <v>341</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>333</v>
+        <v>342</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="1" t="s">
-        <v>334</v>
+        <v>343</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>335</v>
+        <v>344</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>336</v>
+        <v>345</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>337</v>
+        <v>346</v>
       </c>
     </row>
     <row r="21" ht="15.75" customHeight="1"/>

</xml_diff>